<commit_message>
new BAU and blue ammonia inventories
</commit_message>
<xml_diff>
--- a/Raw data/lci-Abhi image SSP2-Base 2020 ammonia and methanol.xlsx
+++ b/Raw data/lci-Abhi image SSP2-Base 2020 ammonia and methanol.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anabera\Desktop\Ongoing projects\Prospective LCA\Raw data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/abhinabera/Desktop/Prospective-LCA/Raw data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEB6CE3E-0E19-4C3E-B243-B0992F63468E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9504D793-11B1-BC45-A4E2-7E56F5CA4F8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="510" windowWidth="28800" windowHeight="17490" activeTab="1" xr2:uid="{79F87D26-5407-4579-9D8D-FA563FE5FD90}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" activeTab="1" xr2:uid="{79F87D26-5407-4579-9D8D-FA563FE5FD90}"/>
   </bookViews>
   <sheets>
     <sheet name="Utilities" sheetId="6" r:id="rId1"/>
@@ -21,12 +21,23 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1150" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1152" uniqueCount="167">
   <si>
     <t>Activity</t>
   </si>
@@ -520,13 +531,13 @@
     <t>market for tap water</t>
   </si>
   <si>
-    <t>ammonia, BAU with CCS</t>
-  </si>
-  <si>
     <t>This is the activity for the production of BAU ammonia with CCS</t>
   </si>
   <si>
     <t>lci-Abhi image SSP2-Base 2020 ammonia and methanol</t>
+  </si>
+  <si>
+    <t>ammonia, blue</t>
   </si>
 </sst>
 </file>
@@ -606,7 +617,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -637,7 +648,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -957,24 +967,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55E8D1F9-2651-4D58-AB8D-D63402B2F76A}">
   <dimension ref="A1:K227"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="70.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.7109375" customWidth="1"/>
-    <col min="3" max="3" width="38.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="25.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="70.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.6640625" customWidth="1"/>
+    <col min="3" max="3" width="38.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="25.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="8" t="s">
         <v>43</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C1" s="9"/>
       <c r="D1" s="10"/>
@@ -983,7 +993,7 @@
       <c r="G1" s="10"/>
       <c r="H1" s="10"/>
     </row>
-    <row r="2" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="3"/>
@@ -993,7 +1003,7 @@
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -1007,7 +1017,7 @@
       <c r="G3" s="6"/>
       <c r="H3" s="6"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
         <v>2</v>
       </c>
@@ -1021,7 +1031,7 @@
       <c r="G4" s="6"/>
       <c r="H4" s="6"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
         <v>3</v>
       </c>
@@ -1035,7 +1045,7 @@
       <c r="G5" s="6"/>
       <c r="H5" s="6"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
         <v>5</v>
       </c>
@@ -1049,7 +1059,7 @@
       <c r="G6" s="6"/>
       <c r="H6" s="6"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
         <v>6</v>
       </c>
@@ -1063,7 +1073,7 @@
       <c r="G7" s="6"/>
       <c r="H7" s="6"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
         <v>8</v>
       </c>
@@ -1077,7 +1087,7 @@
       <c r="G8" s="6"/>
       <c r="H8" s="6"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>10</v>
       </c>
@@ -1089,7 +1099,7 @@
       <c r="G9" s="6"/>
       <c r="H9" s="6"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
         <v>11</v>
       </c>
@@ -1115,7 +1125,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>49</v>
       </c>
@@ -1139,7 +1149,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>51</v>
       </c>
@@ -1163,7 +1173,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>53</v>
       </c>
@@ -1186,7 +1196,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="14" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="3"/>
@@ -1196,7 +1206,7 @@
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>0</v>
       </c>
@@ -1210,7 +1220,7 @@
       <c r="G15" s="6"/>
       <c r="H15" s="6"/>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" s="6" t="s">
         <v>2</v>
       </c>
@@ -1224,7 +1234,7 @@
       <c r="G16" s="6"/>
       <c r="H16" s="6"/>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" s="6" t="s">
         <v>3</v>
       </c>
@@ -1238,7 +1248,7 @@
       <c r="G17" s="6"/>
       <c r="H17" s="6"/>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" s="6" t="s">
         <v>5</v>
       </c>
@@ -1252,7 +1262,7 @@
       <c r="G18" s="6"/>
       <c r="H18" s="6"/>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" s="6" t="s">
         <v>6</v>
       </c>
@@ -1266,7 +1276,7 @@
       <c r="G19" s="6"/>
       <c r="H19" s="6"/>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" s="6" t="s">
         <v>8</v>
       </c>
@@ -1280,7 +1290,7 @@
       <c r="G20" s="6"/>
       <c r="H20" s="6"/>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>10</v>
       </c>
@@ -1292,7 +1302,7 @@
       <c r="G21" s="6"/>
       <c r="H21" s="6"/>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="6" t="s">
         <v>11</v>
       </c>
@@ -1318,7 +1328,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>54</v>
       </c>
@@ -1342,7 +1352,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>56</v>
       </c>
@@ -1366,7 +1376,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>58</v>
       </c>
@@ -1389,7 +1399,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>60</v>
       </c>
@@ -1412,7 +1422,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>53</v>
       </c>
@@ -1435,7 +1445,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
       <c r="C28" s="3"/>
@@ -1445,7 +1455,7 @@
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
         <v>0</v>
       </c>
@@ -1459,7 +1469,7 @@
       <c r="G29" s="6"/>
       <c r="H29" s="6"/>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A30" s="6" t="s">
         <v>2</v>
       </c>
@@ -1473,7 +1483,7 @@
       <c r="G30" s="6"/>
       <c r="H30" s="6"/>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" s="6" t="s">
         <v>3</v>
       </c>
@@ -1487,7 +1497,7 @@
       <c r="G31" s="6"/>
       <c r="H31" s="6"/>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32" s="6" t="s">
         <v>5</v>
       </c>
@@ -1501,7 +1511,7 @@
       <c r="G32" s="6"/>
       <c r="H32" s="6"/>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33" s="6" t="s">
         <v>6</v>
       </c>
@@ -1515,7 +1525,7 @@
       <c r="G33" s="6"/>
       <c r="H33" s="6"/>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A34" s="6" t="s">
         <v>8</v>
       </c>
@@ -1529,7 +1539,7 @@
       <c r="G34" s="6"/>
       <c r="H34" s="6"/>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
         <v>10</v>
       </c>
@@ -1541,7 +1551,7 @@
       <c r="G35" s="6"/>
       <c r="H35" s="6"/>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A36" s="6" t="s">
         <v>11</v>
       </c>
@@ -1567,7 +1577,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>61</v>
       </c>
@@ -1591,7 +1601,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>63</v>
       </c>
@@ -1615,7 +1625,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>65</v>
       </c>
@@ -1638,7 +1648,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>67</v>
       </c>
@@ -1661,7 +1671,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>53</v>
       </c>
@@ -1684,7 +1694,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="3"/>
@@ -1694,7 +1704,7 @@
       <c r="G42" s="2"/>
       <c r="H42" s="2"/>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
         <v>0</v>
       </c>
@@ -1708,7 +1718,7 @@
       <c r="G43" s="6"/>
       <c r="H43" s="6"/>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A44" s="6" t="s">
         <v>2</v>
       </c>
@@ -1722,7 +1732,7 @@
       <c r="G44" s="6"/>
       <c r="H44" s="6"/>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A45" s="6" t="s">
         <v>3</v>
       </c>
@@ -1736,7 +1746,7 @@
       <c r="G45" s="6"/>
       <c r="H45" s="6"/>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A46" s="6" t="s">
         <v>5</v>
       </c>
@@ -1750,7 +1760,7 @@
       <c r="G46" s="6"/>
       <c r="H46" s="6"/>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A47" s="6" t="s">
         <v>6</v>
       </c>
@@ -1764,7 +1774,7 @@
       <c r="G47" s="6"/>
       <c r="H47" s="6"/>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A48" s="6" t="s">
         <v>8</v>
       </c>
@@ -1778,7 +1788,7 @@
       <c r="G48" s="6"/>
       <c r="H48" s="6"/>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
         <v>10</v>
       </c>
@@ -1790,7 +1800,7 @@
       <c r="G49" s="6"/>
       <c r="H49" s="6"/>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A50" s="6" t="s">
         <v>11</v>
       </c>
@@ -1816,7 +1826,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>69</v>
       </c>
@@ -1840,7 +1850,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>51</v>
       </c>
@@ -1864,7 +1874,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>71</v>
       </c>
@@ -1887,7 +1897,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>60</v>
       </c>
@@ -1910,7 +1920,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>53</v>
       </c>
@@ -1933,7 +1943,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A56" s="2"/>
       <c r="B56" s="2"/>
       <c r="C56" s="3"/>
@@ -1943,7 +1953,7 @@
       <c r="G56" s="2"/>
       <c r="H56" s="2"/>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
         <v>0</v>
       </c>
@@ -1957,7 +1967,7 @@
       <c r="G57" s="6"/>
       <c r="H57" s="6"/>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" s="6" t="s">
         <v>2</v>
       </c>
@@ -1971,7 +1981,7 @@
       <c r="G58" s="6"/>
       <c r="H58" s="6"/>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A59" s="6" t="s">
         <v>3</v>
       </c>
@@ -1985,7 +1995,7 @@
       <c r="G59" s="6"/>
       <c r="H59" s="6"/>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A60" s="6" t="s">
         <v>5</v>
       </c>
@@ -1999,7 +2009,7 @@
       <c r="G60" s="6"/>
       <c r="H60" s="6"/>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A61" s="6" t="s">
         <v>6</v>
       </c>
@@ -2013,7 +2023,7 @@
       <c r="G61" s="6"/>
       <c r="H61" s="6"/>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A62" s="6" t="s">
         <v>8</v>
       </c>
@@ -2027,7 +2037,7 @@
       <c r="G62" s="6"/>
       <c r="H62" s="6"/>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A63" s="1" t="s">
         <v>10</v>
       </c>
@@ -2039,7 +2049,7 @@
       <c r="G63" s="6"/>
       <c r="H63" s="6"/>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A64" s="6" t="s">
         <v>11</v>
       </c>
@@ -2065,7 +2075,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>73</v>
       </c>
@@ -2089,7 +2099,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>75</v>
       </c>
@@ -2113,7 +2123,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>60</v>
       </c>
@@ -2136,7 +2146,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>53</v>
       </c>
@@ -2159,7 +2169,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A69" s="2"/>
       <c r="B69" s="2"/>
       <c r="C69" s="3"/>
@@ -2169,7 +2179,7 @@
       <c r="G69" s="2"/>
       <c r="H69" s="2"/>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A70" s="1" t="s">
         <v>0</v>
       </c>
@@ -2183,7 +2193,7 @@
       <c r="G70" s="6"/>
       <c r="H70" s="6"/>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A71" s="6" t="s">
         <v>2</v>
       </c>
@@ -2197,7 +2207,7 @@
       <c r="G71" s="6"/>
       <c r="H71" s="6"/>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A72" s="6" t="s">
         <v>3</v>
       </c>
@@ -2211,7 +2221,7 @@
       <c r="G72" s="6"/>
       <c r="H72" s="6"/>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A73" s="6" t="s">
         <v>5</v>
       </c>
@@ -2225,7 +2235,7 @@
       <c r="G73" s="6"/>
       <c r="H73" s="6"/>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A74" s="6" t="s">
         <v>6</v>
       </c>
@@ -2239,7 +2249,7 @@
       <c r="G74" s="6"/>
       <c r="H74" s="6"/>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A75" s="6" t="s">
         <v>8</v>
       </c>
@@ -2253,7 +2263,7 @@
       <c r="G75" s="6"/>
       <c r="H75" s="6"/>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76" s="1" t="s">
         <v>10</v>
       </c>
@@ -2265,7 +2275,7 @@
       <c r="G76" s="6"/>
       <c r="H76" s="6"/>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A77" s="6" t="s">
         <v>11</v>
       </c>
@@ -2291,7 +2301,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>76</v>
       </c>
@@ -2315,7 +2325,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>63</v>
       </c>
@@ -2339,7 +2349,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>78</v>
       </c>
@@ -2363,7 +2373,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>60</v>
       </c>
@@ -2386,7 +2396,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>53</v>
       </c>
@@ -2409,7 +2419,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A83" s="2"/>
       <c r="B83" s="2"/>
       <c r="C83" s="3"/>
@@ -2419,7 +2429,7 @@
       <c r="G83" s="2"/>
       <c r="H83" s="2"/>
     </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A84" s="1" t="s">
         <v>0</v>
       </c>
@@ -2433,7 +2443,7 @@
       <c r="G84" s="6"/>
       <c r="H84" s="6"/>
     </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A85" s="6" t="s">
         <v>2</v>
       </c>
@@ -2447,7 +2457,7 @@
       <c r="G85" s="6"/>
       <c r="H85" s="6"/>
     </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A86" s="6" t="s">
         <v>3</v>
       </c>
@@ -2461,7 +2471,7 @@
       <c r="G86" s="6"/>
       <c r="H86" s="6"/>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A87" s="6" t="s">
         <v>5</v>
       </c>
@@ -2475,7 +2485,7 @@
       <c r="G87" s="6"/>
       <c r="H87" s="6"/>
     </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A88" s="6" t="s">
         <v>6</v>
       </c>
@@ -2489,7 +2499,7 @@
       <c r="G88" s="6"/>
       <c r="H88" s="6"/>
     </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A89" s="6" t="s">
         <v>8</v>
       </c>
@@ -2503,7 +2513,7 @@
       <c r="G89" s="6"/>
       <c r="H89" s="6"/>
     </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A90" s="1" t="s">
         <v>10</v>
       </c>
@@ -2515,7 +2525,7 @@
       <c r="G90" s="6"/>
       <c r="H90" s="6"/>
     </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A91" s="6" t="s">
         <v>11</v>
       </c>
@@ -2541,7 +2551,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>80</v>
       </c>
@@ -2565,7 +2575,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>75</v>
       </c>
@@ -2589,7 +2599,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>60</v>
       </c>
@@ -2612,7 +2622,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>53</v>
       </c>
@@ -2635,7 +2645,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A96" s="2"/>
       <c r="B96" s="2"/>
       <c r="C96" s="3"/>
@@ -2645,7 +2655,7 @@
       <c r="G96" s="2"/>
       <c r="H96" s="2"/>
     </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A97" s="1" t="s">
         <v>0</v>
       </c>
@@ -2659,7 +2669,7 @@
       <c r="G97" s="6"/>
       <c r="H97" s="6"/>
     </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A98" s="6" t="s">
         <v>2</v>
       </c>
@@ -2673,7 +2683,7 @@
       <c r="G98" s="6"/>
       <c r="H98" s="6"/>
     </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A99" s="6" t="s">
         <v>3</v>
       </c>
@@ -2687,7 +2697,7 @@
       <c r="G99" s="6"/>
       <c r="H99" s="6"/>
     </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A100" s="6" t="s">
         <v>5</v>
       </c>
@@ -2701,7 +2711,7 @@
       <c r="G100" s="6"/>
       <c r="H100" s="6"/>
     </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A101" s="6" t="s">
         <v>6</v>
       </c>
@@ -2715,7 +2725,7 @@
       <c r="G101" s="6"/>
       <c r="H101" s="6"/>
     </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A102" s="6" t="s">
         <v>8</v>
       </c>
@@ -2729,7 +2739,7 @@
       <c r="G102" s="6"/>
       <c r="H102" s="6"/>
     </row>
-    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A103" s="1" t="s">
         <v>10</v>
       </c>
@@ -2741,7 +2751,7 @@
       <c r="G103" s="6"/>
       <c r="H103" s="6"/>
     </row>
-    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A104" s="6" t="s">
         <v>11</v>
       </c>
@@ -2767,7 +2777,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>161</v>
       </c>
@@ -2791,7 +2801,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>49</v>
       </c>
@@ -2815,7 +2825,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="107" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>54</v>
       </c>
@@ -2839,7 +2849,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="108" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>61</v>
       </c>
@@ -2863,7 +2873,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>69</v>
       </c>
@@ -2887,7 +2897,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="110" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>73</v>
       </c>
@@ -2911,7 +2921,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="111" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>76</v>
       </c>
@@ -2935,7 +2945,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="112" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>80</v>
       </c>
@@ -2959,7 +2969,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="113" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A113" s="2"/>
       <c r="B113" s="2"/>
       <c r="C113" s="3"/>
@@ -2969,7 +2979,7 @@
       <c r="G113" s="2"/>
       <c r="H113" s="2"/>
     </row>
-    <row r="114" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A114" s="1" t="s">
         <v>0</v>
       </c>
@@ -2983,7 +2993,7 @@
       <c r="G114" s="6"/>
       <c r="H114" s="6"/>
     </row>
-    <row r="115" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A115" s="6" t="s">
         <v>2</v>
       </c>
@@ -2997,7 +3007,7 @@
       <c r="G115" s="6"/>
       <c r="H115" s="6"/>
     </row>
-    <row r="116" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A116" s="6" t="s">
         <v>3</v>
       </c>
@@ -3011,7 +3021,7 @@
       <c r="G116" s="6"/>
       <c r="H116" s="6"/>
     </row>
-    <row r="117" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A117" s="6" t="s">
         <v>5</v>
       </c>
@@ -3025,7 +3035,7 @@
       <c r="G117" s="6"/>
       <c r="H117" s="6"/>
     </row>
-    <row r="118" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A118" s="6" t="s">
         <v>6</v>
       </c>
@@ -3039,7 +3049,7 @@
       <c r="G118" s="6"/>
       <c r="H118" s="6"/>
     </row>
-    <row r="119" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A119" s="6" t="s">
         <v>8</v>
       </c>
@@ -3053,7 +3063,7 @@
       <c r="G119" s="6"/>
       <c r="H119" s="6"/>
     </row>
-    <row r="120" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A120" s="1" t="s">
         <v>10</v>
       </c>
@@ -3065,7 +3075,7 @@
       <c r="G120" s="6"/>
       <c r="H120" s="6"/>
     </row>
-    <row r="121" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A121" s="6" t="s">
         <v>11</v>
       </c>
@@ -3091,7 +3101,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="122" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
         <v>83</v>
       </c>
@@ -3115,7 +3125,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="123" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
         <v>86</v>
       </c>
@@ -3140,7 +3150,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="124" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
         <v>46</v>
       </c>
@@ -3165,7 +3175,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="125" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
         <v>88</v>
       </c>
@@ -3190,7 +3200,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="126" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
         <v>90</v>
       </c>
@@ -3215,7 +3225,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="127" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
         <v>35</v>
       </c>
@@ -3236,7 +3246,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="128" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
         <v>92</v>
       </c>
@@ -3257,7 +3267,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="129" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
         <v>93</v>
       </c>
@@ -3281,7 +3291,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="130" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A130" s="2"/>
       <c r="B130" s="2"/>
       <c r="C130" s="3"/>
@@ -3291,7 +3301,7 @@
       <c r="G130" s="2"/>
       <c r="H130" s="2"/>
     </row>
-    <row r="131" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A131" s="1" t="s">
         <v>0</v>
       </c>
@@ -3305,7 +3315,7 @@
       <c r="G131" s="6"/>
       <c r="H131" s="6"/>
     </row>
-    <row r="132" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A132" s="6" t="s">
         <v>2</v>
       </c>
@@ -3319,7 +3329,7 @@
       <c r="G132" s="6"/>
       <c r="H132" s="6"/>
     </row>
-    <row r="133" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A133" s="6" t="s">
         <v>3</v>
       </c>
@@ -3333,7 +3343,7 @@
       <c r="G133" s="6"/>
       <c r="H133" s="6"/>
     </row>
-    <row r="134" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A134" s="6" t="s">
         <v>5</v>
       </c>
@@ -3347,7 +3357,7 @@
       <c r="G134" s="6"/>
       <c r="H134" s="6"/>
     </row>
-    <row r="135" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A135" s="6" t="s">
         <v>6</v>
       </c>
@@ -3361,7 +3371,7 @@
       <c r="G135" s="6"/>
       <c r="H135" s="6"/>
     </row>
-    <row r="136" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A136" s="6" t="s">
         <v>8</v>
       </c>
@@ -3375,7 +3385,7 @@
       <c r="G136" s="6"/>
       <c r="H136" s="6"/>
     </row>
-    <row r="137" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A137" s="1" t="s">
         <v>10</v>
       </c>
@@ -3387,7 +3397,7 @@
       <c r="G137" s="6"/>
       <c r="H137" s="6"/>
     </row>
-    <row r="138" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A138" s="6" t="s">
         <v>11</v>
       </c>
@@ -3413,7 +3423,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="139" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
         <v>95</v>
       </c>
@@ -3437,7 +3447,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="140" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
         <v>98</v>
       </c>
@@ -3458,7 +3468,7 @@
       </c>
       <c r="K140" s="12"/>
     </row>
-    <row r="141" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
         <v>37</v>
       </c>
@@ -3479,7 +3489,7 @@
       </c>
       <c r="K141" s="12"/>
     </row>
-    <row r="142" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
         <v>99</v>
       </c>
@@ -3500,7 +3510,7 @@
       </c>
       <c r="K142" s="12"/>
     </row>
-    <row r="143" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A143" t="s">
         <v>100</v>
       </c>
@@ -3521,7 +3531,7 @@
       </c>
       <c r="K143" s="12"/>
     </row>
-    <row r="144" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A144" t="s">
         <v>101</v>
       </c>
@@ -3542,7 +3552,7 @@
       </c>
       <c r="K144" s="12"/>
     </row>
-    <row r="145" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A145" t="s">
         <v>102</v>
       </c>
@@ -3563,7 +3573,7 @@
       </c>
       <c r="K145" s="12"/>
     </row>
-    <row r="146" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A146" t="s">
         <v>103</v>
       </c>
@@ -3584,7 +3594,7 @@
       </c>
       <c r="K146" s="12"/>
     </row>
-    <row r="147" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A147" t="s">
         <v>104</v>
       </c>
@@ -3605,7 +3615,7 @@
       </c>
       <c r="K147" s="12"/>
     </row>
-    <row r="148" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A148" t="s">
         <v>105</v>
       </c>
@@ -3626,7 +3636,7 @@
       </c>
       <c r="K148" s="12"/>
     </row>
-    <row r="149" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A149" t="s">
         <v>106</v>
       </c>
@@ -3647,7 +3657,7 @@
       </c>
       <c r="K149" s="12"/>
     </row>
-    <row r="150" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A150" t="s">
         <v>107</v>
       </c>
@@ -3668,7 +3678,7 @@
       </c>
       <c r="K150" s="12"/>
     </row>
-    <row r="151" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A151" t="s">
         <v>108</v>
       </c>
@@ -3689,7 +3699,7 @@
       </c>
       <c r="K151" s="12"/>
     </row>
-    <row r="152" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A152" t="s">
         <v>109</v>
       </c>
@@ -3710,7 +3720,7 @@
       </c>
       <c r="K152" s="12"/>
     </row>
-    <row r="153" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A153" t="s">
         <v>110</v>
       </c>
@@ -3731,7 +3741,7 @@
       </c>
       <c r="K153" s="12"/>
     </row>
-    <row r="154" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A154" t="s">
         <v>111</v>
       </c>
@@ -3752,7 +3762,7 @@
       </c>
       <c r="K154" s="12"/>
     </row>
-    <row r="155" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A155" t="s">
         <v>112</v>
       </c>
@@ -3773,7 +3783,7 @@
       </c>
       <c r="K155" s="12"/>
     </row>
-    <row r="156" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A156" t="s">
         <v>113</v>
       </c>
@@ -3794,7 +3804,7 @@
       </c>
       <c r="K156" s="12"/>
     </row>
-    <row r="157" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A157" t="s">
         <v>114</v>
       </c>
@@ -3815,7 +3825,7 @@
       </c>
       <c r="K157" s="12"/>
     </row>
-    <row r="158" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A158" t="s">
         <v>115</v>
       </c>
@@ -3836,7 +3846,7 @@
       </c>
       <c r="K158" s="12"/>
     </row>
-    <row r="159" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A159" t="s">
         <v>116</v>
       </c>
@@ -3857,7 +3867,7 @@
       </c>
       <c r="K159" s="12"/>
     </row>
-    <row r="160" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A160" s="2"/>
       <c r="B160" s="2"/>
       <c r="C160" s="3"/>
@@ -3867,7 +3877,7 @@
       <c r="G160" s="2"/>
       <c r="H160" s="2"/>
     </row>
-    <row r="161" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A161" s="1" t="s">
         <v>0</v>
       </c>
@@ -3882,7 +3892,7 @@
       <c r="H161" s="6"/>
       <c r="I161" s="6"/>
     </row>
-    <row r="162" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A162" s="6" t="s">
         <v>2</v>
       </c>
@@ -3897,7 +3907,7 @@
       <c r="H162" s="6"/>
       <c r="I162" s="6"/>
     </row>
-    <row r="163" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A163" s="6" t="s">
         <v>3</v>
       </c>
@@ -3912,7 +3922,7 @@
       <c r="H163" s="6"/>
       <c r="I163" s="6"/>
     </row>
-    <row r="164" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A164" s="6" t="s">
         <v>5</v>
       </c>
@@ -3927,7 +3937,7 @@
       <c r="H164" s="6"/>
       <c r="I164" s="6"/>
     </row>
-    <row r="165" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A165" s="6" t="s">
         <v>6</v>
       </c>
@@ -3942,7 +3952,7 @@
       <c r="H165" s="6"/>
       <c r="I165" s="6"/>
     </row>
-    <row r="166" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A166" s="6" t="s">
         <v>8</v>
       </c>
@@ -3957,7 +3967,7 @@
       <c r="H166" s="6"/>
       <c r="I166" s="6"/>
     </row>
-    <row r="167" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A167" s="1" t="s">
         <v>10</v>
       </c>
@@ -3970,7 +3980,7 @@
       <c r="H167" s="6"/>
       <c r="I167" s="6"/>
     </row>
-    <row r="168" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A168" s="6" t="s">
         <v>11</v>
       </c>
@@ -3997,7 +4007,7 @@
       </c>
       <c r="I168" s="6"/>
     </row>
-    <row r="169" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A169" s="6" t="s">
         <v>29</v>
       </c>
@@ -4020,7 +4030,7 @@
       <c r="H169" s="6"/>
       <c r="I169" s="6"/>
     </row>
-    <row r="170" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A170" s="6" t="s">
         <v>122</v>
       </c>
@@ -4044,7 +4054,7 @@
       <c r="I170" s="6"/>
       <c r="K170" s="12"/>
     </row>
-    <row r="171" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A171" s="6" t="s">
         <v>125</v>
       </c>
@@ -4068,7 +4078,7 @@
       <c r="I171" s="6"/>
       <c r="K171" s="12"/>
     </row>
-    <row r="172" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A172" s="6" t="s">
         <v>127</v>
       </c>
@@ -4092,7 +4102,7 @@
       <c r="I172" s="6"/>
       <c r="K172" s="12"/>
     </row>
-    <row r="173" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A173" s="6" t="s">
         <v>129</v>
       </c>
@@ -4116,7 +4126,7 @@
       <c r="I173" s="6"/>
       <c r="K173" s="12"/>
     </row>
-    <row r="174" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A174" s="6" t="s">
         <v>120</v>
       </c>
@@ -4142,7 +4152,7 @@
       <c r="I174" s="6"/>
       <c r="K174" s="12"/>
     </row>
-    <row r="175" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A175" s="6" t="s">
         <v>130</v>
       </c>
@@ -4168,7 +4178,7 @@
       <c r="I175" s="6"/>
       <c r="K175" s="12"/>
     </row>
-    <row r="176" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A176" s="6" t="s">
         <v>132</v>
       </c>
@@ -4194,7 +4204,7 @@
       <c r="I176" s="6"/>
       <c r="K176" s="12"/>
     </row>
-    <row r="177" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A177" s="6" t="s">
         <v>134</v>
       </c>
@@ -4220,7 +4230,7 @@
       <c r="I177" s="6"/>
       <c r="K177" s="12"/>
     </row>
-    <row r="178" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A178" s="6" t="s">
         <v>136</v>
       </c>
@@ -4246,7 +4256,7 @@
       <c r="I178" s="6"/>
       <c r="K178" s="12"/>
     </row>
-    <row r="179" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A179" s="6" t="s">
         <v>137</v>
       </c>
@@ -4272,7 +4282,7 @@
       <c r="I179" s="6"/>
       <c r="K179" s="12"/>
     </row>
-    <row r="180" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A180" s="6" t="s">
         <v>138</v>
       </c>
@@ -4298,7 +4308,7 @@
       <c r="I180" s="6"/>
       <c r="K180" s="12"/>
     </row>
-    <row r="181" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A181" s="6" t="s">
         <v>141</v>
       </c>
@@ -4324,7 +4334,7 @@
       <c r="I181" s="6"/>
       <c r="K181" s="12"/>
     </row>
-    <row r="182" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A182" s="6" t="s">
         <v>144</v>
       </c>
@@ -4350,7 +4360,7 @@
       <c r="I182" s="6"/>
       <c r="K182" s="12"/>
     </row>
-    <row r="183" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A183" s="6" t="s">
         <v>146</v>
       </c>
@@ -4376,7 +4386,7 @@
       <c r="I183" s="6"/>
       <c r="K183" s="12"/>
     </row>
-    <row r="184" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A184" s="6" t="s">
         <v>148</v>
       </c>
@@ -4402,7 +4412,7 @@
       <c r="I184" s="6"/>
       <c r="K184" s="12"/>
     </row>
-    <row r="185" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A185" s="6" t="s">
         <v>150</v>
       </c>
@@ -4428,7 +4438,7 @@
       <c r="I185" s="6"/>
       <c r="K185" s="12"/>
     </row>
-    <row r="186" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A186" s="6" t="s">
         <v>152</v>
       </c>
@@ -4454,7 +4464,7 @@
       <c r="I186" s="6"/>
       <c r="K186" s="12"/>
     </row>
-    <row r="187" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A187" s="2"/>
       <c r="B187" s="2"/>
       <c r="C187" s="3"/>
@@ -4465,7 +4475,7 @@
       <c r="H187" s="2"/>
       <c r="K187" s="12"/>
     </row>
-    <row r="188" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A188" s="1" t="s">
         <v>0</v>
       </c>
@@ -4480,7 +4490,7 @@
       <c r="H188" s="6"/>
       <c r="K188" s="12"/>
     </row>
-    <row r="189" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A189" s="6" t="s">
         <v>2</v>
       </c>
@@ -4495,7 +4505,7 @@
       <c r="H189" s="6"/>
       <c r="K189" s="12"/>
     </row>
-    <row r="190" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A190" s="6" t="s">
         <v>3</v>
       </c>
@@ -4509,7 +4519,7 @@
       <c r="G190" s="6"/>
       <c r="H190" s="6"/>
     </row>
-    <row r="191" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A191" s="6" t="s">
         <v>5</v>
       </c>
@@ -4523,7 +4533,7 @@
       <c r="G191" s="6"/>
       <c r="H191" s="6"/>
     </row>
-    <row r="192" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A192" s="6" t="s">
         <v>6</v>
       </c>
@@ -4537,7 +4547,7 @@
       <c r="G192" s="6"/>
       <c r="H192" s="6"/>
     </row>
-    <row r="193" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A193" s="6" t="s">
         <v>8</v>
       </c>
@@ -4551,7 +4561,7 @@
       <c r="G193" s="6"/>
       <c r="H193" s="6"/>
     </row>
-    <row r="194" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A194" s="1" t="s">
         <v>10</v>
       </c>
@@ -4563,7 +4573,7 @@
       <c r="G194" s="6"/>
       <c r="H194" s="6"/>
     </row>
-    <row r="195" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A195" s="6" t="s">
         <v>11</v>
       </c>
@@ -4589,7 +4599,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="196" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A196" s="6" t="s">
         <v>119</v>
       </c>
@@ -4613,7 +4623,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="197" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A197" s="6" t="s">
         <v>120</v>
       </c>
@@ -4637,7 +4647,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="198" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A198" t="s">
         <v>53</v>
       </c>
@@ -4661,7 +4671,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="199" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A199" t="s">
         <v>29</v>
       </c>
@@ -4684,7 +4694,7 @@
       </c>
       <c r="H199" s="6"/>
     </row>
-    <row r="200" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A200" s="2"/>
       <c r="B200" s="2"/>
       <c r="C200" s="3"/>
@@ -4694,7 +4704,7 @@
       <c r="G200" s="2"/>
       <c r="H200" s="2"/>
     </row>
-    <row r="201" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A201" s="1" t="s">
         <v>0</v>
       </c>
@@ -4708,7 +4718,7 @@
       <c r="G201" s="6"/>
       <c r="H201" s="6"/>
     </row>
-    <row r="202" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A202" s="6" t="s">
         <v>2</v>
       </c>
@@ -4722,7 +4732,7 @@
       <c r="G202" s="6"/>
       <c r="H202" s="6"/>
     </row>
-    <row r="203" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A203" s="6" t="s">
         <v>3</v>
       </c>
@@ -4736,7 +4746,7 @@
       <c r="G203" s="6"/>
       <c r="H203" s="6"/>
     </row>
-    <row r="204" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A204" s="6" t="s">
         <v>5</v>
       </c>
@@ -4750,7 +4760,7 @@
       <c r="G204" s="6"/>
       <c r="H204" s="6"/>
     </row>
-    <row r="205" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A205" s="6" t="s">
         <v>6</v>
       </c>
@@ -4764,7 +4774,7 @@
       <c r="G205" s="6"/>
       <c r="H205" s="6"/>
     </row>
-    <row r="206" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A206" s="6" t="s">
         <v>8</v>
       </c>
@@ -4778,7 +4788,7 @@
       <c r="G206" s="6"/>
       <c r="H206" s="6"/>
     </row>
-    <row r="207" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A207" s="1" t="s">
         <v>10</v>
       </c>
@@ -4790,7 +4800,7 @@
       <c r="G207" s="6"/>
       <c r="H207" s="6"/>
     </row>
-    <row r="208" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A208" s="6" t="s">
         <v>11</v>
       </c>
@@ -4816,7 +4826,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="209" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A209" s="6" t="s">
         <v>156</v>
       </c>
@@ -4840,7 +4850,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="210" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A210" s="6" t="s">
         <v>120</v>
       </c>
@@ -4864,7 +4874,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="211" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A211" t="s">
         <v>53</v>
       </c>
@@ -4888,7 +4898,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="212" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A212" t="s">
         <v>29</v>
       </c>
@@ -4911,7 +4921,7 @@
       </c>
       <c r="H212" s="6"/>
     </row>
-    <row r="213" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A213" s="2"/>
       <c r="B213" s="2"/>
       <c r="C213" s="3"/>
@@ -4921,7 +4931,7 @@
       <c r="G213" s="2"/>
       <c r="H213" s="2"/>
     </row>
-    <row r="214" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A214" s="1" t="s">
         <v>0</v>
       </c>
@@ -4935,7 +4945,7 @@
       <c r="G214" s="6"/>
       <c r="H214" s="6"/>
     </row>
-    <row r="215" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A215" s="6" t="s">
         <v>2</v>
       </c>
@@ -4949,7 +4959,7 @@
       <c r="G215" s="6"/>
       <c r="H215" s="6"/>
     </row>
-    <row r="216" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A216" s="6" t="s">
         <v>3</v>
       </c>
@@ -4963,7 +4973,7 @@
       <c r="G216" s="6"/>
       <c r="H216" s="6"/>
     </row>
-    <row r="217" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A217" s="6" t="s">
         <v>5</v>
       </c>
@@ -4977,7 +4987,7 @@
       <c r="G217" s="6"/>
       <c r="H217" s="6"/>
     </row>
-    <row r="218" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A218" s="6" t="s">
         <v>6</v>
       </c>
@@ -4991,7 +5001,7 @@
       <c r="G218" s="6"/>
       <c r="H218" s="6"/>
     </row>
-    <row r="219" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A219" s="6" t="s">
         <v>8</v>
       </c>
@@ -5005,7 +5015,7 @@
       <c r="G219" s="6"/>
       <c r="H219" s="6"/>
     </row>
-    <row r="220" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A220" s="1" t="s">
         <v>10</v>
       </c>
@@ -5017,7 +5027,7 @@
       <c r="G220" s="6"/>
       <c r="H220" s="6"/>
     </row>
-    <row r="221" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A221" s="6" t="s">
         <v>11</v>
       </c>
@@ -5043,7 +5053,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="222" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A222" s="6" t="s">
         <v>157</v>
       </c>
@@ -5067,7 +5077,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="223" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A223" t="s">
         <v>83</v>
       </c>
@@ -5091,7 +5101,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="224" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A224" s="6" t="s">
         <v>156</v>
       </c>
@@ -5115,7 +5125,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="225" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A225" s="6" t="s">
         <v>159</v>
       </c>
@@ -5139,7 +5149,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="226" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A226" t="s">
         <v>53</v>
       </c>
@@ -5162,7 +5172,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="227" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A227" t="s">
         <v>29</v>
       </c>
@@ -5193,18 +5203,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD968991-55C9-4627-9323-29F50518FFEB}">
   <dimension ref="A1:H65"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="86.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="86.5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="38.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.5" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="25.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="25.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5218,7 +5228,7 @@
       <c r="G1" s="6"/>
       <c r="H1" s="6"/>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
         <v>2</v>
       </c>
@@ -5232,7 +5242,7 @@
       <c r="G2" s="6"/>
       <c r="H2" s="6"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>3</v>
       </c>
@@ -5246,7 +5256,7 @@
       <c r="G3" s="6"/>
       <c r="H3" s="6"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
         <v>5</v>
       </c>
@@ -5260,7 +5270,7 @@
       <c r="G4" s="6"/>
       <c r="H4" s="6"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
         <v>6</v>
       </c>
@@ -5274,7 +5284,7 @@
       <c r="G5" s="6"/>
       <c r="H5" s="6"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
         <v>8</v>
       </c>
@@ -5288,7 +5298,7 @@
       <c r="G6" s="6"/>
       <c r="H6" s="6"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>10</v>
       </c>
@@ -5300,7 +5310,7 @@
       <c r="G7" s="6"/>
       <c r="H7" s="6"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
         <v>11</v>
       </c>
@@ -5326,7 +5336,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>1</v>
       </c>
@@ -5350,7 +5360,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>45</v>
       </c>
@@ -5374,7 +5384,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>163</v>
       </c>
@@ -5397,7 +5407,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>47</v>
       </c>
@@ -5420,7 +5430,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>27</v>
       </c>
@@ -5444,7 +5454,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>161</v>
       </c>
@@ -5468,7 +5478,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>83</v>
       </c>
@@ -5492,7 +5502,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>90</v>
       </c>
@@ -5515,7 +5525,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>32</v>
       </c>
@@ -5528,14 +5538,14 @@
       <c r="E17" t="s">
         <v>21</v>
       </c>
-      <c r="F17" s="16" t="s">
+      <c r="F17" t="s">
         <v>33</v>
       </c>
       <c r="G17" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>95</v>
       </c>
@@ -5559,7 +5569,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>53</v>
       </c>
@@ -5582,7 +5592,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" s="12" t="s">
         <v>34</v>
       </c>
@@ -5602,7 +5612,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>35</v>
       </c>
@@ -5622,7 +5632,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>98</v>
       </c>
@@ -5642,7 +5652,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>99</v>
       </c>
@@ -5663,7 +5673,7 @@
       </c>
       <c r="H23" s="12"/>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>29</v>
       </c>
@@ -5684,7 +5694,7 @@
       </c>
       <c r="H24" s="12"/>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>37</v>
       </c>
@@ -5704,18 +5714,19 @@
         <v>31</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>38</v>
       </c>
-      <c r="B26" s="17">
-        <v>149</v>
+      <c r="B26" s="16">
+        <f>149/1000</f>
+        <v>0.14899999999999999</v>
       </c>
       <c r="C26" s="15" t="s">
         <v>30</v>
       </c>
       <c r="E26" t="s">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="F26" t="s">
         <v>39</v>
@@ -5724,7 +5735,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>36</v>
       </c>
@@ -5744,7 +5755,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>92</v>
       </c>
@@ -5764,18 +5775,19 @@
         <v>31</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>38</v>
       </c>
-      <c r="B29" s="17">
-        <v>422</v>
+      <c r="B29" s="16">
+        <f>422/1000</f>
+        <v>0.42199999999999999</v>
       </c>
       <c r="C29" s="15" t="s">
         <v>30</v>
       </c>
       <c r="E29" t="s">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="F29" s="15" t="s">
         <v>40</v>
@@ -5784,7 +5796,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>152</v>
       </c>
@@ -5808,7 +5820,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>162</v>
       </c>
@@ -5818,6 +5830,9 @@
       <c r="C31" t="s">
         <v>18</v>
       </c>
+      <c r="D31" t="s">
+        <v>19</v>
+      </c>
       <c r="E31" s="5" t="s">
         <v>21</v>
       </c>
@@ -5829,7 +5844,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32" s="3"/>
@@ -5839,23 +5854,23 @@
       <c r="G32" s="2"/>
       <c r="H32" s="2"/>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>2</v>
       </c>
       <c r="B34" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>3</v>
       </c>
@@ -5863,7 +5878,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>5</v>
       </c>
@@ -5871,7 +5886,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>6</v>
       </c>
@@ -5879,7 +5894,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>8</v>
       </c>
@@ -5887,12 +5902,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>11</v>
       </c>
@@ -5918,9 +5933,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B41" s="4">
         <v>1</v>
@@ -5941,7 +5956,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>45</v>
       </c>
@@ -5965,7 +5980,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>163</v>
       </c>
@@ -5988,7 +6003,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>47</v>
       </c>
@@ -6011,7 +6026,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>27</v>
       </c>
@@ -6035,7 +6050,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>161</v>
       </c>
@@ -6059,7 +6074,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>83</v>
       </c>
@@ -6083,7 +6098,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A48" s="6" t="s">
         <v>119</v>
       </c>
@@ -6107,7 +6122,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>32</v>
       </c>
@@ -6120,14 +6135,14 @@
       <c r="E49" t="s">
         <v>21</v>
       </c>
-      <c r="F49" s="16" t="s">
+      <c r="F49" t="s">
         <v>33</v>
       </c>
       <c r="G49" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>95</v>
       </c>
@@ -6151,7 +6166,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>53</v>
       </c>
@@ -6174,7 +6189,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A52" s="6" t="s">
         <v>157</v>
       </c>
@@ -6198,7 +6213,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A53" s="12" t="s">
         <v>34</v>
       </c>
@@ -6218,7 +6233,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>35</v>
       </c>
@@ -6238,7 +6253,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>98</v>
       </c>
@@ -6258,7 +6273,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>99</v>
       </c>
@@ -6279,7 +6294,7 @@
       </c>
       <c r="H56" s="12"/>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>29</v>
       </c>
@@ -6300,7 +6315,7 @@
       </c>
       <c r="H57" s="12"/>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>37</v>
       </c>
@@ -6320,18 +6335,19 @@
         <v>31</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>38</v>
       </c>
-      <c r="B59" s="17">
-        <v>153.04</v>
+      <c r="B59" s="16">
+        <f>153.04/1000</f>
+        <v>0.15303999999999998</v>
       </c>
       <c r="C59" s="15" t="s">
         <v>30</v>
       </c>
       <c r="E59" t="s">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="F59" t="s">
         <v>39</v>
@@ -6340,7 +6356,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>36</v>
       </c>
@@ -6360,7 +6376,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>92</v>
       </c>
@@ -6380,18 +6396,19 @@
         <v>31</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>38</v>
       </c>
-      <c r="B62" s="17">
-        <v>419</v>
+      <c r="B62" s="16">
+        <f>419/1000</f>
+        <v>0.41899999999999998</v>
       </c>
       <c r="C62" s="15" t="s">
         <v>30</v>
       </c>
       <c r="E62" t="s">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="F62" s="15" t="s">
         <v>40</v>
@@ -6400,7 +6417,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>152</v>
       </c>
@@ -6424,7 +6441,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>162</v>
       </c>
@@ -6434,6 +6451,9 @@
       <c r="C64" t="s">
         <v>18</v>
       </c>
+      <c r="D64" t="s">
+        <v>19</v>
+      </c>
       <c r="E64" s="5" t="s">
         <v>21</v>
       </c>
@@ -6445,7 +6465,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A65" s="6"/>
       <c r="B65" s="11"/>
       <c r="C65" s="6"/>

</xml_diff>

<commit_message>
BAU and blue methanol inventories
</commit_message>
<xml_diff>
--- a/Raw data/lci-Abhi image SSP2-Base 2020 ammonia and methanol.xlsx
+++ b/Raw data/lci-Abhi image SSP2-Base 2020 ammonia and methanol.xlsx
@@ -1,43 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20404"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/abhinabera/Desktop/Prospective-LCA/Raw data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anabera\Desktop\Ongoing projects\Prospective LCA\Raw data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9504D793-11B1-BC45-A4E2-7E56F5CA4F8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B92D1BC2-4EC1-441E-9595-2C63B1EBA2E2}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" activeTab="1" xr2:uid="{79F87D26-5407-4579-9D8D-FA563FE5FD90}"/>
+    <workbookView xWindow="0" yWindow="495" windowWidth="28800" windowHeight="17505" activeTab="2" xr2:uid="{79F87D26-5407-4579-9D8D-FA563FE5FD90}"/>
   </bookViews>
   <sheets>
     <sheet name="Utilities" sheetId="6" r:id="rId1"/>
     <sheet name="Ammonia" sheetId="5" r:id="rId2"/>
+    <sheet name="Methanol" sheetId="7" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1152" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1452" uniqueCount="178">
   <si>
     <t>Activity</t>
   </si>
@@ -538,6 +528,39 @@
   </si>
   <si>
     <t>ammonia, blue</t>
+  </si>
+  <si>
+    <t>methanol, BAU</t>
+  </si>
+  <si>
+    <t>This is the activity for 1 kg of BAU methanol</t>
+  </si>
+  <si>
+    <t>methanol, Abhi</t>
+  </si>
+  <si>
+    <t>market for steam, in chemical industry</t>
+  </si>
+  <si>
+    <t>steam, in chemical industry</t>
+  </si>
+  <si>
+    <t>market for cooling energy</t>
+  </si>
+  <si>
+    <t>cooling energy</t>
+  </si>
+  <si>
+    <t>Oxygen</t>
+  </si>
+  <si>
+    <t>Methanol</t>
+  </si>
+  <si>
+    <t>methanol, blue</t>
+  </si>
+  <si>
+    <t>This is the activity for 1 kg of blue methanol</t>
   </si>
 </sst>
 </file>
@@ -967,19 +990,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55E8D1F9-2651-4D58-AB8D-D63402B2F76A}">
   <dimension ref="A1:K227"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="70.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.6640625" customWidth="1"/>
-    <col min="3" max="3" width="38.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="25.1640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="70.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.7109375" customWidth="1"/>
+    <col min="3" max="3" width="38.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="25.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>43</v>
       </c>
@@ -993,7 +1016,7 @@
       <c r="G1" s="10"/>
       <c r="H1" s="10"/>
     </row>
-    <row r="2" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="3"/>
@@ -1003,7 +1026,7 @@
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -1017,7 +1040,7 @@
       <c r="G3" s="6"/>
       <c r="H3" s="6"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>2</v>
       </c>
@@ -1031,7 +1054,7 @@
       <c r="G4" s="6"/>
       <c r="H4" s="6"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>3</v>
       </c>
@@ -1045,7 +1068,7 @@
       <c r="G5" s="6"/>
       <c r="H5" s="6"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>5</v>
       </c>
@@ -1059,7 +1082,7 @@
       <c r="G6" s="6"/>
       <c r="H6" s="6"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>6</v>
       </c>
@@ -1073,7 +1096,7 @@
       <c r="G7" s="6"/>
       <c r="H7" s="6"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>8</v>
       </c>
@@ -1087,7 +1110,7 @@
       <c r="G8" s="6"/>
       <c r="H8" s="6"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>10</v>
       </c>
@@ -1099,7 +1122,7 @@
       <c r="G9" s="6"/>
       <c r="H9" s="6"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>11</v>
       </c>
@@ -1125,7 +1148,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>49</v>
       </c>
@@ -1149,7 +1172,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>51</v>
       </c>
@@ -1173,7 +1196,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>53</v>
       </c>
@@ -1196,7 +1219,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="14" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="3"/>
@@ -1206,7 +1229,7 @@
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>0</v>
       </c>
@@ -1220,7 +1243,7 @@
       <c r="G15" s="6"/>
       <c r="H15" s="6"/>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>2</v>
       </c>
@@ -1234,7 +1257,7 @@
       <c r="G16" s="6"/>
       <c r="H16" s="6"/>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>3</v>
       </c>
@@ -1248,7 +1271,7 @@
       <c r="G17" s="6"/>
       <c r="H17" s="6"/>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>5</v>
       </c>
@@ -1262,7 +1285,7 @@
       <c r="G18" s="6"/>
       <c r="H18" s="6"/>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>6</v>
       </c>
@@ -1276,7 +1299,7 @@
       <c r="G19" s="6"/>
       <c r="H19" s="6"/>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>8</v>
       </c>
@@ -1290,7 +1313,7 @@
       <c r="G20" s="6"/>
       <c r="H20" s="6"/>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>10</v>
       </c>
@@ -1302,7 +1325,7 @@
       <c r="G21" s="6"/>
       <c r="H21" s="6"/>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>11</v>
       </c>
@@ -1328,7 +1351,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>54</v>
       </c>
@@ -1352,7 +1375,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>56</v>
       </c>
@@ -1376,7 +1399,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>58</v>
       </c>
@@ -1399,7 +1422,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>60</v>
       </c>
@@ -1422,7 +1445,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>53</v>
       </c>
@@ -1445,7 +1468,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
       <c r="C28" s="3"/>
@@ -1455,7 +1478,7 @@
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>0</v>
       </c>
@@ -1469,7 +1492,7 @@
       <c r="G29" s="6"/>
       <c r="H29" s="6"/>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
         <v>2</v>
       </c>
@@ -1483,7 +1506,7 @@
       <c r="G30" s="6"/>
       <c r="H30" s="6"/>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
         <v>3</v>
       </c>
@@ -1497,7 +1520,7 @@
       <c r="G31" s="6"/>
       <c r="H31" s="6"/>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
         <v>5</v>
       </c>
@@ -1511,7 +1534,7 @@
       <c r="G32" s="6"/>
       <c r="H32" s="6"/>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
         <v>6</v>
       </c>
@@ -1525,7 +1548,7 @@
       <c r="G33" s="6"/>
       <c r="H33" s="6"/>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
         <v>8</v>
       </c>
@@ -1539,7 +1562,7 @@
       <c r="G34" s="6"/>
       <c r="H34" s="6"/>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>10</v>
       </c>
@@ -1551,7 +1574,7 @@
       <c r="G35" s="6"/>
       <c r="H35" s="6"/>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
         <v>11</v>
       </c>
@@ -1577,7 +1600,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>61</v>
       </c>
@@ -1601,7 +1624,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>63</v>
       </c>
@@ -1625,7 +1648,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>65</v>
       </c>
@@ -1648,7 +1671,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>67</v>
       </c>
@@ -1671,7 +1694,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>53</v>
       </c>
@@ -1694,7 +1717,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="3"/>
@@ -1704,7 +1727,7 @@
       <c r="G42" s="2"/>
       <c r="H42" s="2"/>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>0</v>
       </c>
@@ -1718,7 +1741,7 @@
       <c r="G43" s="6"/>
       <c r="H43" s="6"/>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="6" t="s">
         <v>2</v>
       </c>
@@ -1732,7 +1755,7 @@
       <c r="G44" s="6"/>
       <c r="H44" s="6"/>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="6" t="s">
         <v>3</v>
       </c>
@@ -1746,7 +1769,7 @@
       <c r="G45" s="6"/>
       <c r="H45" s="6"/>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" s="6" t="s">
         <v>5</v>
       </c>
@@ -1760,7 +1783,7 @@
       <c r="G46" s="6"/>
       <c r="H46" s="6"/>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" s="6" t="s">
         <v>6</v>
       </c>
@@ -1774,7 +1797,7 @@
       <c r="G47" s="6"/>
       <c r="H47" s="6"/>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" s="6" t="s">
         <v>8</v>
       </c>
@@ -1788,7 +1811,7 @@
       <c r="G48" s="6"/>
       <c r="H48" s="6"/>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>10</v>
       </c>
@@ -1800,7 +1823,7 @@
       <c r="G49" s="6"/>
       <c r="H49" s="6"/>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" s="6" t="s">
         <v>11</v>
       </c>
@@ -1826,7 +1849,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>69</v>
       </c>
@@ -1850,7 +1873,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>51</v>
       </c>
@@ -1874,7 +1897,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>71</v>
       </c>
@@ -1897,7 +1920,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>60</v>
       </c>
@@ -1920,7 +1943,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>53</v>
       </c>
@@ -1943,7 +1966,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" s="2"/>
       <c r="B56" s="2"/>
       <c r="C56" s="3"/>
@@ -1953,7 +1976,7 @@
       <c r="G56" s="2"/>
       <c r="H56" s="2"/>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>0</v>
       </c>
@@ -1967,7 +1990,7 @@
       <c r="G57" s="6"/>
       <c r="H57" s="6"/>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" s="6" t="s">
         <v>2</v>
       </c>
@@ -1981,7 +2004,7 @@
       <c r="G58" s="6"/>
       <c r="H58" s="6"/>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" s="6" t="s">
         <v>3</v>
       </c>
@@ -1995,7 +2018,7 @@
       <c r="G59" s="6"/>
       <c r="H59" s="6"/>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" s="6" t="s">
         <v>5</v>
       </c>
@@ -2009,7 +2032,7 @@
       <c r="G60" s="6"/>
       <c r="H60" s="6"/>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" s="6" t="s">
         <v>6</v>
       </c>
@@ -2023,7 +2046,7 @@
       <c r="G61" s="6"/>
       <c r="H61" s="6"/>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" s="6" t="s">
         <v>8</v>
       </c>
@@ -2037,7 +2060,7 @@
       <c r="G62" s="6"/>
       <c r="H62" s="6"/>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>10</v>
       </c>
@@ -2049,7 +2072,7 @@
       <c r="G63" s="6"/>
       <c r="H63" s="6"/>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" s="6" t="s">
         <v>11</v>
       </c>
@@ -2075,7 +2098,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>73</v>
       </c>
@@ -2099,7 +2122,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>75</v>
       </c>
@@ -2123,7 +2146,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>60</v>
       </c>
@@ -2146,7 +2169,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>53</v>
       </c>
@@ -2169,7 +2192,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" s="2"/>
       <c r="B69" s="2"/>
       <c r="C69" s="3"/>
@@ -2179,7 +2202,7 @@
       <c r="G69" s="2"/>
       <c r="H69" s="2"/>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>0</v>
       </c>
@@ -2193,7 +2216,7 @@
       <c r="G70" s="6"/>
       <c r="H70" s="6"/>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" s="6" t="s">
         <v>2</v>
       </c>
@@ -2207,7 +2230,7 @@
       <c r="G71" s="6"/>
       <c r="H71" s="6"/>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72" s="6" t="s">
         <v>3</v>
       </c>
@@ -2221,7 +2244,7 @@
       <c r="G72" s="6"/>
       <c r="H72" s="6"/>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73" s="6" t="s">
         <v>5</v>
       </c>
@@ -2235,7 +2258,7 @@
       <c r="G73" s="6"/>
       <c r="H73" s="6"/>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74" s="6" t="s">
         <v>6</v>
       </c>
@@ -2249,7 +2272,7 @@
       <c r="G74" s="6"/>
       <c r="H74" s="6"/>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75" s="6" t="s">
         <v>8</v>
       </c>
@@ -2263,7 +2286,7 @@
       <c r="G75" s="6"/>
       <c r="H75" s="6"/>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
         <v>10</v>
       </c>
@@ -2275,7 +2298,7 @@
       <c r="G76" s="6"/>
       <c r="H76" s="6"/>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77" s="6" t="s">
         <v>11</v>
       </c>
@@ -2301,7 +2324,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>76</v>
       </c>
@@ -2325,7 +2348,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>63</v>
       </c>
@@ -2349,7 +2372,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>78</v>
       </c>
@@ -2373,7 +2396,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>60</v>
       </c>
@@ -2396,7 +2419,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>53</v>
       </c>
@@ -2419,7 +2442,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A83" s="2"/>
       <c r="B83" s="2"/>
       <c r="C83" s="3"/>
@@ -2429,7 +2452,7 @@
       <c r="G83" s="2"/>
       <c r="H83" s="2"/>
     </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
         <v>0</v>
       </c>
@@ -2443,7 +2466,7 @@
       <c r="G84" s="6"/>
       <c r="H84" s="6"/>
     </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A85" s="6" t="s">
         <v>2</v>
       </c>
@@ -2457,7 +2480,7 @@
       <c r="G85" s="6"/>
       <c r="H85" s="6"/>
     </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A86" s="6" t="s">
         <v>3</v>
       </c>
@@ -2471,7 +2494,7 @@
       <c r="G86" s="6"/>
       <c r="H86" s="6"/>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A87" s="6" t="s">
         <v>5</v>
       </c>
@@ -2485,7 +2508,7 @@
       <c r="G87" s="6"/>
       <c r="H87" s="6"/>
     </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A88" s="6" t="s">
         <v>6</v>
       </c>
@@ -2499,7 +2522,7 @@
       <c r="G88" s="6"/>
       <c r="H88" s="6"/>
     </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A89" s="6" t="s">
         <v>8</v>
       </c>
@@ -2513,7 +2536,7 @@
       <c r="G89" s="6"/>
       <c r="H89" s="6"/>
     </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
         <v>10</v>
       </c>
@@ -2525,7 +2548,7 @@
       <c r="G90" s="6"/>
       <c r="H90" s="6"/>
     </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A91" s="6" t="s">
         <v>11</v>
       </c>
@@ -2551,7 +2574,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>80</v>
       </c>
@@ -2575,7 +2598,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>75</v>
       </c>
@@ -2599,7 +2622,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>60</v>
       </c>
@@ -2622,7 +2645,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>53</v>
       </c>
@@ -2645,7 +2668,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A96" s="2"/>
       <c r="B96" s="2"/>
       <c r="C96" s="3"/>
@@ -2655,7 +2678,7 @@
       <c r="G96" s="2"/>
       <c r="H96" s="2"/>
     </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A97" s="1" t="s">
         <v>0</v>
       </c>
@@ -2669,7 +2692,7 @@
       <c r="G97" s="6"/>
       <c r="H97" s="6"/>
     </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A98" s="6" t="s">
         <v>2</v>
       </c>
@@ -2683,7 +2706,7 @@
       <c r="G98" s="6"/>
       <c r="H98" s="6"/>
     </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A99" s="6" t="s">
         <v>3</v>
       </c>
@@ -2697,7 +2720,7 @@
       <c r="G99" s="6"/>
       <c r="H99" s="6"/>
     </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A100" s="6" t="s">
         <v>5</v>
       </c>
@@ -2711,7 +2734,7 @@
       <c r="G100" s="6"/>
       <c r="H100" s="6"/>
     </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A101" s="6" t="s">
         <v>6</v>
       </c>
@@ -2725,7 +2748,7 @@
       <c r="G101" s="6"/>
       <c r="H101" s="6"/>
     </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A102" s="6" t="s">
         <v>8</v>
       </c>
@@ -2739,7 +2762,7 @@
       <c r="G102" s="6"/>
       <c r="H102" s="6"/>
     </row>
-    <row r="103" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A103" s="1" t="s">
         <v>10</v>
       </c>
@@ -2751,7 +2774,7 @@
       <c r="G103" s="6"/>
       <c r="H103" s="6"/>
     </row>
-    <row r="104" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A104" s="6" t="s">
         <v>11</v>
       </c>
@@ -2777,7 +2800,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>161</v>
       </c>
@@ -2801,7 +2824,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>49</v>
       </c>
@@ -2825,7 +2848,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="107" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>54</v>
       </c>
@@ -2849,7 +2872,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="108" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>61</v>
       </c>
@@ -2873,7 +2896,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="109" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>69</v>
       </c>
@@ -2897,7 +2920,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="110" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>73</v>
       </c>
@@ -2921,7 +2944,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="111" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>76</v>
       </c>
@@ -2945,7 +2968,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="112" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>80</v>
       </c>
@@ -2969,7 +2992,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="113" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A113" s="2"/>
       <c r="B113" s="2"/>
       <c r="C113" s="3"/>
@@ -2979,7 +3002,7 @@
       <c r="G113" s="2"/>
       <c r="H113" s="2"/>
     </row>
-    <row r="114" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A114" s="1" t="s">
         <v>0</v>
       </c>
@@ -2993,7 +3016,7 @@
       <c r="G114" s="6"/>
       <c r="H114" s="6"/>
     </row>
-    <row r="115" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A115" s="6" t="s">
         <v>2</v>
       </c>
@@ -3007,7 +3030,7 @@
       <c r="G115" s="6"/>
       <c r="H115" s="6"/>
     </row>
-    <row r="116" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A116" s="6" t="s">
         <v>3</v>
       </c>
@@ -3021,7 +3044,7 @@
       <c r="G116" s="6"/>
       <c r="H116" s="6"/>
     </row>
-    <row r="117" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A117" s="6" t="s">
         <v>5</v>
       </c>
@@ -3035,7 +3058,7 @@
       <c r="G117" s="6"/>
       <c r="H117" s="6"/>
     </row>
-    <row r="118" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A118" s="6" t="s">
         <v>6</v>
       </c>
@@ -3049,7 +3072,7 @@
       <c r="G118" s="6"/>
       <c r="H118" s="6"/>
     </row>
-    <row r="119" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A119" s="6" t="s">
         <v>8</v>
       </c>
@@ -3063,7 +3086,7 @@
       <c r="G119" s="6"/>
       <c r="H119" s="6"/>
     </row>
-    <row r="120" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A120" s="1" t="s">
         <v>10</v>
       </c>
@@ -3075,7 +3098,7 @@
       <c r="G120" s="6"/>
       <c r="H120" s="6"/>
     </row>
-    <row r="121" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A121" s="6" t="s">
         <v>11</v>
       </c>
@@ -3101,7 +3124,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="122" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>83</v>
       </c>
@@ -3125,7 +3148,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="123" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>86</v>
       </c>
@@ -3150,7 +3173,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="124" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>46</v>
       </c>
@@ -3175,7 +3198,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="125" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>88</v>
       </c>
@@ -3200,7 +3223,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="126" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>90</v>
       </c>
@@ -3225,7 +3248,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="127" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>35</v>
       </c>
@@ -3246,7 +3269,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="128" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>92</v>
       </c>
@@ -3267,7 +3290,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="129" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>93</v>
       </c>
@@ -3291,7 +3314,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="130" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A130" s="2"/>
       <c r="B130" s="2"/>
       <c r="C130" s="3"/>
@@ -3301,7 +3324,7 @@
       <c r="G130" s="2"/>
       <c r="H130" s="2"/>
     </row>
-    <row r="131" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A131" s="1" t="s">
         <v>0</v>
       </c>
@@ -3315,7 +3338,7 @@
       <c r="G131" s="6"/>
       <c r="H131" s="6"/>
     </row>
-    <row r="132" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A132" s="6" t="s">
         <v>2</v>
       </c>
@@ -3329,7 +3352,7 @@
       <c r="G132" s="6"/>
       <c r="H132" s="6"/>
     </row>
-    <row r="133" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A133" s="6" t="s">
         <v>3</v>
       </c>
@@ -3343,7 +3366,7 @@
       <c r="G133" s="6"/>
       <c r="H133" s="6"/>
     </row>
-    <row r="134" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A134" s="6" t="s">
         <v>5</v>
       </c>
@@ -3357,7 +3380,7 @@
       <c r="G134" s="6"/>
       <c r="H134" s="6"/>
     </row>
-    <row r="135" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A135" s="6" t="s">
         <v>6</v>
       </c>
@@ -3371,7 +3394,7 @@
       <c r="G135" s="6"/>
       <c r="H135" s="6"/>
     </row>
-    <row r="136" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A136" s="6" t="s">
         <v>8</v>
       </c>
@@ -3385,7 +3408,7 @@
       <c r="G136" s="6"/>
       <c r="H136" s="6"/>
     </row>
-    <row r="137" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A137" s="1" t="s">
         <v>10</v>
       </c>
@@ -3397,7 +3420,7 @@
       <c r="G137" s="6"/>
       <c r="H137" s="6"/>
     </row>
-    <row r="138" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A138" s="6" t="s">
         <v>11</v>
       </c>
@@ -3423,7 +3446,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="139" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>95</v>
       </c>
@@ -3447,7 +3470,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="140" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>98</v>
       </c>
@@ -3468,7 +3491,7 @@
       </c>
       <c r="K140" s="12"/>
     </row>
-    <row r="141" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>37</v>
       </c>
@@ -3489,7 +3512,7 @@
       </c>
       <c r="K141" s="12"/>
     </row>
-    <row r="142" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>99</v>
       </c>
@@ -3510,7 +3533,7 @@
       </c>
       <c r="K142" s="12"/>
     </row>
-    <row r="143" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>100</v>
       </c>
@@ -3531,7 +3554,7 @@
       </c>
       <c r="K143" s="12"/>
     </row>
-    <row r="144" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>101</v>
       </c>
@@ -3552,7 +3575,7 @@
       </c>
       <c r="K144" s="12"/>
     </row>
-    <row r="145" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>102</v>
       </c>
@@ -3573,7 +3596,7 @@
       </c>
       <c r="K145" s="12"/>
     </row>
-    <row r="146" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>103</v>
       </c>
@@ -3594,7 +3617,7 @@
       </c>
       <c r="K146" s="12"/>
     </row>
-    <row r="147" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>104</v>
       </c>
@@ -3615,7 +3638,7 @@
       </c>
       <c r="K147" s="12"/>
     </row>
-    <row r="148" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>105</v>
       </c>
@@ -3636,7 +3659,7 @@
       </c>
       <c r="K148" s="12"/>
     </row>
-    <row r="149" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>106</v>
       </c>
@@ -3657,7 +3680,7 @@
       </c>
       <c r="K149" s="12"/>
     </row>
-    <row r="150" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>107</v>
       </c>
@@ -3678,7 +3701,7 @@
       </c>
       <c r="K150" s="12"/>
     </row>
-    <row r="151" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>108</v>
       </c>
@@ -3699,7 +3722,7 @@
       </c>
       <c r="K151" s="12"/>
     </row>
-    <row r="152" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>109</v>
       </c>
@@ -3720,7 +3743,7 @@
       </c>
       <c r="K152" s="12"/>
     </row>
-    <row r="153" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>110</v>
       </c>
@@ -3741,7 +3764,7 @@
       </c>
       <c r="K153" s="12"/>
     </row>
-    <row r="154" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>111</v>
       </c>
@@ -3762,7 +3785,7 @@
       </c>
       <c r="K154" s="12"/>
     </row>
-    <row r="155" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>112</v>
       </c>
@@ -3783,7 +3806,7 @@
       </c>
       <c r="K155" s="12"/>
     </row>
-    <row r="156" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>113</v>
       </c>
@@ -3804,7 +3827,7 @@
       </c>
       <c r="K156" s="12"/>
     </row>
-    <row r="157" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>114</v>
       </c>
@@ -3825,7 +3848,7 @@
       </c>
       <c r="K157" s="12"/>
     </row>
-    <row r="158" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>115</v>
       </c>
@@ -3846,7 +3869,7 @@
       </c>
       <c r="K158" s="12"/>
     </row>
-    <row r="159" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>116</v>
       </c>
@@ -3867,7 +3890,7 @@
       </c>
       <c r="K159" s="12"/>
     </row>
-    <row r="160" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A160" s="2"/>
       <c r="B160" s="2"/>
       <c r="C160" s="3"/>
@@ -3877,7 +3900,7 @@
       <c r="G160" s="2"/>
       <c r="H160" s="2"/>
     </row>
-    <row r="161" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A161" s="1" t="s">
         <v>0</v>
       </c>
@@ -3892,7 +3915,7 @@
       <c r="H161" s="6"/>
       <c r="I161" s="6"/>
     </row>
-    <row r="162" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A162" s="6" t="s">
         <v>2</v>
       </c>
@@ -3907,7 +3930,7 @@
       <c r="H162" s="6"/>
       <c r="I162" s="6"/>
     </row>
-    <row r="163" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A163" s="6" t="s">
         <v>3</v>
       </c>
@@ -3922,7 +3945,7 @@
       <c r="H163" s="6"/>
       <c r="I163" s="6"/>
     </row>
-    <row r="164" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A164" s="6" t="s">
         <v>5</v>
       </c>
@@ -3937,7 +3960,7 @@
       <c r="H164" s="6"/>
       <c r="I164" s="6"/>
     </row>
-    <row r="165" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A165" s="6" t="s">
         <v>6</v>
       </c>
@@ -3952,7 +3975,7 @@
       <c r="H165" s="6"/>
       <c r="I165" s="6"/>
     </row>
-    <row r="166" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A166" s="6" t="s">
         <v>8</v>
       </c>
@@ -3967,7 +3990,7 @@
       <c r="H166" s="6"/>
       <c r="I166" s="6"/>
     </row>
-    <row r="167" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A167" s="1" t="s">
         <v>10</v>
       </c>
@@ -3980,7 +4003,7 @@
       <c r="H167" s="6"/>
       <c r="I167" s="6"/>
     </row>
-    <row r="168" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A168" s="6" t="s">
         <v>11</v>
       </c>
@@ -4007,7 +4030,7 @@
       </c>
       <c r="I168" s="6"/>
     </row>
-    <row r="169" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A169" s="6" t="s">
         <v>29</v>
       </c>
@@ -4030,7 +4053,7 @@
       <c r="H169" s="6"/>
       <c r="I169" s="6"/>
     </row>
-    <row r="170" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A170" s="6" t="s">
         <v>122</v>
       </c>
@@ -4054,7 +4077,7 @@
       <c r="I170" s="6"/>
       <c r="K170" s="12"/>
     </row>
-    <row r="171" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A171" s="6" t="s">
         <v>125</v>
       </c>
@@ -4078,7 +4101,7 @@
       <c r="I171" s="6"/>
       <c r="K171" s="12"/>
     </row>
-    <row r="172" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A172" s="6" t="s">
         <v>127</v>
       </c>
@@ -4102,7 +4125,7 @@
       <c r="I172" s="6"/>
       <c r="K172" s="12"/>
     </row>
-    <row r="173" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A173" s="6" t="s">
         <v>129</v>
       </c>
@@ -4126,7 +4149,7 @@
       <c r="I173" s="6"/>
       <c r="K173" s="12"/>
     </row>
-    <row r="174" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A174" s="6" t="s">
         <v>120</v>
       </c>
@@ -4152,7 +4175,7 @@
       <c r="I174" s="6"/>
       <c r="K174" s="12"/>
     </row>
-    <row r="175" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A175" s="6" t="s">
         <v>130</v>
       </c>
@@ -4178,7 +4201,7 @@
       <c r="I175" s="6"/>
       <c r="K175" s="12"/>
     </row>
-    <row r="176" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A176" s="6" t="s">
         <v>132</v>
       </c>
@@ -4204,7 +4227,7 @@
       <c r="I176" s="6"/>
       <c r="K176" s="12"/>
     </row>
-    <row r="177" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A177" s="6" t="s">
         <v>134</v>
       </c>
@@ -4230,7 +4253,7 @@
       <c r="I177" s="6"/>
       <c r="K177" s="12"/>
     </row>
-    <row r="178" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A178" s="6" t="s">
         <v>136</v>
       </c>
@@ -4256,7 +4279,7 @@
       <c r="I178" s="6"/>
       <c r="K178" s="12"/>
     </row>
-    <row r="179" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A179" s="6" t="s">
         <v>137</v>
       </c>
@@ -4282,7 +4305,7 @@
       <c r="I179" s="6"/>
       <c r="K179" s="12"/>
     </row>
-    <row r="180" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A180" s="6" t="s">
         <v>138</v>
       </c>
@@ -4308,7 +4331,7 @@
       <c r="I180" s="6"/>
       <c r="K180" s="12"/>
     </row>
-    <row r="181" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A181" s="6" t="s">
         <v>141</v>
       </c>
@@ -4334,7 +4357,7 @@
       <c r="I181" s="6"/>
       <c r="K181" s="12"/>
     </row>
-    <row r="182" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A182" s="6" t="s">
         <v>144</v>
       </c>
@@ -4360,7 +4383,7 @@
       <c r="I182" s="6"/>
       <c r="K182" s="12"/>
     </row>
-    <row r="183" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A183" s="6" t="s">
         <v>146</v>
       </c>
@@ -4386,7 +4409,7 @@
       <c r="I183" s="6"/>
       <c r="K183" s="12"/>
     </row>
-    <row r="184" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A184" s="6" t="s">
         <v>148</v>
       </c>
@@ -4412,7 +4435,7 @@
       <c r="I184" s="6"/>
       <c r="K184" s="12"/>
     </row>
-    <row r="185" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A185" s="6" t="s">
         <v>150</v>
       </c>
@@ -4438,7 +4461,7 @@
       <c r="I185" s="6"/>
       <c r="K185" s="12"/>
     </row>
-    <row r="186" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A186" s="6" t="s">
         <v>152</v>
       </c>
@@ -4464,7 +4487,7 @@
       <c r="I186" s="6"/>
       <c r="K186" s="12"/>
     </row>
-    <row r="187" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A187" s="2"/>
       <c r="B187" s="2"/>
       <c r="C187" s="3"/>
@@ -4475,7 +4498,7 @@
       <c r="H187" s="2"/>
       <c r="K187" s="12"/>
     </row>
-    <row r="188" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A188" s="1" t="s">
         <v>0</v>
       </c>
@@ -4490,7 +4513,7 @@
       <c r="H188" s="6"/>
       <c r="K188" s="12"/>
     </row>
-    <row r="189" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A189" s="6" t="s">
         <v>2</v>
       </c>
@@ -4505,7 +4528,7 @@
       <c r="H189" s="6"/>
       <c r="K189" s="12"/>
     </row>
-    <row r="190" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A190" s="6" t="s">
         <v>3</v>
       </c>
@@ -4519,7 +4542,7 @@
       <c r="G190" s="6"/>
       <c r="H190" s="6"/>
     </row>
-    <row r="191" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A191" s="6" t="s">
         <v>5</v>
       </c>
@@ -4533,7 +4556,7 @@
       <c r="G191" s="6"/>
       <c r="H191" s="6"/>
     </row>
-    <row r="192" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A192" s="6" t="s">
         <v>6</v>
       </c>
@@ -4547,7 +4570,7 @@
       <c r="G192" s="6"/>
       <c r="H192" s="6"/>
     </row>
-    <row r="193" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A193" s="6" t="s">
         <v>8</v>
       </c>
@@ -4561,7 +4584,7 @@
       <c r="G193" s="6"/>
       <c r="H193" s="6"/>
     </row>
-    <row r="194" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A194" s="1" t="s">
         <v>10</v>
       </c>
@@ -4573,7 +4596,7 @@
       <c r="G194" s="6"/>
       <c r="H194" s="6"/>
     </row>
-    <row r="195" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A195" s="6" t="s">
         <v>11</v>
       </c>
@@ -4599,7 +4622,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="196" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A196" s="6" t="s">
         <v>119</v>
       </c>
@@ -4623,7 +4646,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="197" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A197" s="6" t="s">
         <v>120</v>
       </c>
@@ -4647,7 +4670,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="198" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
         <v>53</v>
       </c>
@@ -4671,7 +4694,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="199" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
         <v>29</v>
       </c>
@@ -4694,7 +4717,7 @@
       </c>
       <c r="H199" s="6"/>
     </row>
-    <row r="200" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A200" s="2"/>
       <c r="B200" s="2"/>
       <c r="C200" s="3"/>
@@ -4704,7 +4727,7 @@
       <c r="G200" s="2"/>
       <c r="H200" s="2"/>
     </row>
-    <row r="201" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A201" s="1" t="s">
         <v>0</v>
       </c>
@@ -4718,7 +4741,7 @@
       <c r="G201" s="6"/>
       <c r="H201" s="6"/>
     </row>
-    <row r="202" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="202" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A202" s="6" t="s">
         <v>2</v>
       </c>
@@ -4732,7 +4755,7 @@
       <c r="G202" s="6"/>
       <c r="H202" s="6"/>
     </row>
-    <row r="203" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A203" s="6" t="s">
         <v>3</v>
       </c>
@@ -4746,7 +4769,7 @@
       <c r="G203" s="6"/>
       <c r="H203" s="6"/>
     </row>
-    <row r="204" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A204" s="6" t="s">
         <v>5</v>
       </c>
@@ -4760,7 +4783,7 @@
       <c r="G204" s="6"/>
       <c r="H204" s="6"/>
     </row>
-    <row r="205" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A205" s="6" t="s">
         <v>6</v>
       </c>
@@ -4774,7 +4797,7 @@
       <c r="G205" s="6"/>
       <c r="H205" s="6"/>
     </row>
-    <row r="206" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="206" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A206" s="6" t="s">
         <v>8</v>
       </c>
@@ -4788,7 +4811,7 @@
       <c r="G206" s="6"/>
       <c r="H206" s="6"/>
     </row>
-    <row r="207" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A207" s="1" t="s">
         <v>10</v>
       </c>
@@ -4800,7 +4823,7 @@
       <c r="G207" s="6"/>
       <c r="H207" s="6"/>
     </row>
-    <row r="208" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A208" s="6" t="s">
         <v>11</v>
       </c>
@@ -4826,7 +4849,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="209" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A209" s="6" t="s">
         <v>156</v>
       </c>
@@ -4850,7 +4873,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="210" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A210" s="6" t="s">
         <v>120</v>
       </c>
@@ -4874,7 +4897,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="211" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
         <v>53</v>
       </c>
@@ -4898,7 +4921,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="212" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
         <v>29</v>
       </c>
@@ -4921,7 +4944,7 @@
       </c>
       <c r="H212" s="6"/>
     </row>
-    <row r="213" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A213" s="2"/>
       <c r="B213" s="2"/>
       <c r="C213" s="3"/>
@@ -4931,7 +4954,7 @@
       <c r="G213" s="2"/>
       <c r="H213" s="2"/>
     </row>
-    <row r="214" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A214" s="1" t="s">
         <v>0</v>
       </c>
@@ -4945,7 +4968,7 @@
       <c r="G214" s="6"/>
       <c r="H214" s="6"/>
     </row>
-    <row r="215" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="215" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A215" s="6" t="s">
         <v>2</v>
       </c>
@@ -4959,7 +4982,7 @@
       <c r="G215" s="6"/>
       <c r="H215" s="6"/>
     </row>
-    <row r="216" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="216" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A216" s="6" t="s">
         <v>3</v>
       </c>
@@ -4973,7 +4996,7 @@
       <c r="G216" s="6"/>
       <c r="H216" s="6"/>
     </row>
-    <row r="217" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="217" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A217" s="6" t="s">
         <v>5</v>
       </c>
@@ -4987,7 +5010,7 @@
       <c r="G217" s="6"/>
       <c r="H217" s="6"/>
     </row>
-    <row r="218" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="218" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A218" s="6" t="s">
         <v>6</v>
       </c>
@@ -5001,7 +5024,7 @@
       <c r="G218" s="6"/>
       <c r="H218" s="6"/>
     </row>
-    <row r="219" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="219" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A219" s="6" t="s">
         <v>8</v>
       </c>
@@ -5015,7 +5038,7 @@
       <c r="G219" s="6"/>
       <c r="H219" s="6"/>
     </row>
-    <row r="220" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="220" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A220" s="1" t="s">
         <v>10</v>
       </c>
@@ -5027,7 +5050,7 @@
       <c r="G220" s="6"/>
       <c r="H220" s="6"/>
     </row>
-    <row r="221" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="221" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A221" s="6" t="s">
         <v>11</v>
       </c>
@@ -5053,7 +5076,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="222" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="222" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A222" s="6" t="s">
         <v>157</v>
       </c>
@@ -5077,7 +5100,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="223" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="223" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
         <v>83</v>
       </c>
@@ -5101,7 +5124,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="224" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="224" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A224" s="6" t="s">
         <v>156</v>
       </c>
@@ -5125,7 +5148,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="225" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="225" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A225" s="6" t="s">
         <v>159</v>
       </c>
@@ -5149,7 +5172,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="226" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="226" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
         <v>53</v>
       </c>
@@ -5172,7 +5195,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="227" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="227" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
         <v>29</v>
       </c>
@@ -5203,18 +5226,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD968991-55C9-4627-9323-29F50518FFEB}">
   <dimension ref="A1:H65"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="86.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="86.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="38.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.42578125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="25.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="25.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5228,7 +5251,7 @@
       <c r="G1" s="6"/>
       <c r="H1" s="6"/>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>2</v>
       </c>
@@ -5242,7 +5265,7 @@
       <c r="G2" s="6"/>
       <c r="H2" s="6"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>3</v>
       </c>
@@ -5256,7 +5279,7 @@
       <c r="G3" s="6"/>
       <c r="H3" s="6"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>5</v>
       </c>
@@ -5270,7 +5293,7 @@
       <c r="G4" s="6"/>
       <c r="H4" s="6"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>6</v>
       </c>
@@ -5284,7 +5307,7 @@
       <c r="G5" s="6"/>
       <c r="H5" s="6"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>8</v>
       </c>
@@ -5298,7 +5321,7 @@
       <c r="G6" s="6"/>
       <c r="H6" s="6"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>10</v>
       </c>
@@ -5310,7 +5333,7 @@
       <c r="G7" s="6"/>
       <c r="H7" s="6"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>11</v>
       </c>
@@ -5336,7 +5359,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>1</v>
       </c>
@@ -5360,7 +5383,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>45</v>
       </c>
@@ -5384,7 +5407,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>163</v>
       </c>
@@ -5407,7 +5430,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>47</v>
       </c>
@@ -5430,7 +5453,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>27</v>
       </c>
@@ -5454,7 +5477,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>161</v>
       </c>
@@ -5478,7 +5501,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>83</v>
       </c>
@@ -5502,7 +5525,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>90</v>
       </c>
@@ -5525,7 +5548,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>32</v>
       </c>
@@ -5545,7 +5568,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>95</v>
       </c>
@@ -5569,7 +5592,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>53</v>
       </c>
@@ -5592,7 +5615,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="12" t="s">
         <v>34</v>
       </c>
@@ -5612,7 +5635,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>35</v>
       </c>
@@ -5632,7 +5655,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>98</v>
       </c>
@@ -5652,7 +5675,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>99</v>
       </c>
@@ -5673,7 +5696,7 @@
       </c>
       <c r="H23" s="12"/>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>29</v>
       </c>
@@ -5694,7 +5717,7 @@
       </c>
       <c r="H24" s="12"/>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>37</v>
       </c>
@@ -5714,7 +5737,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>38</v>
       </c>
@@ -5735,7 +5758,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>36</v>
       </c>
@@ -5755,7 +5778,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>92</v>
       </c>
@@ -5775,7 +5798,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>38</v>
       </c>
@@ -5796,7 +5819,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>152</v>
       </c>
@@ -5820,7 +5843,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>162</v>
       </c>
@@ -5844,7 +5867,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32" s="3"/>
@@ -5854,7 +5877,7 @@
       <c r="G32" s="2"/>
       <c r="H32" s="2"/>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>0</v>
       </c>
@@ -5862,7 +5885,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>2</v>
       </c>
@@ -5870,7 +5893,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>3</v>
       </c>
@@ -5878,7 +5901,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>5</v>
       </c>
@@ -5886,7 +5909,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>6</v>
       </c>
@@ -5894,7 +5917,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>8</v>
       </c>
@@ -5902,12 +5925,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>11</v>
       </c>
@@ -5933,7 +5956,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>166</v>
       </c>
@@ -5956,7 +5979,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>45</v>
       </c>
@@ -5980,7 +6003,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>163</v>
       </c>
@@ -6003,7 +6026,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>47</v>
       </c>
@@ -6026,7 +6049,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>27</v>
       </c>
@@ -6050,7 +6073,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>161</v>
       </c>
@@ -6074,7 +6097,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>83</v>
       </c>
@@ -6098,7 +6121,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" s="6" t="s">
         <v>119</v>
       </c>
@@ -6122,7 +6145,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>32</v>
       </c>
@@ -6142,7 +6165,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>95</v>
       </c>
@@ -6166,7 +6189,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>53</v>
       </c>
@@ -6189,7 +6212,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" s="6" t="s">
         <v>157</v>
       </c>
@@ -6213,7 +6236,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" s="12" t="s">
         <v>34</v>
       </c>
@@ -6233,7 +6256,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>35</v>
       </c>
@@ -6253,7 +6276,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>98</v>
       </c>
@@ -6273,7 +6296,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>99</v>
       </c>
@@ -6294,7 +6317,7 @@
       </c>
       <c r="H56" s="12"/>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>29</v>
       </c>
@@ -6315,7 +6338,7 @@
       </c>
       <c r="H57" s="12"/>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>37</v>
       </c>
@@ -6335,7 +6358,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>38</v>
       </c>
@@ -6356,7 +6379,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>36</v>
       </c>
@@ -6376,7 +6399,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>92</v>
       </c>
@@ -6396,7 +6419,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>38</v>
       </c>
@@ -6417,7 +6440,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>152</v>
       </c>
@@ -6441,7 +6464,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>162</v>
       </c>
@@ -6465,7 +6488,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" s="6"/>
       <c r="B65" s="11"/>
       <c r="C65" s="6"/>
@@ -6478,4 +6501,1360 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79B42196-31F0-452D-ABB3-56E1539B21DD}">
+  <dimension ref="A1:L77"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="86.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="25.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>168</v>
+      </c>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="7"/>
+      <c r="I2" s="6"/>
+      <c r="J2" s="6"/>
+      <c r="L2" s="6"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="6">
+        <v>1</v>
+      </c>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" t="s">
+        <v>169</v>
+      </c>
+      <c r="C5" s="6"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6"/>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="6"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
+      <c r="F6" s="6"/>
+      <c r="G6" s="6"/>
+      <c r="H6" s="6"/>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H8" s="6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>167</v>
+      </c>
+      <c r="B9" s="7">
+        <v>1</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E9" t="s">
+        <v>9</v>
+      </c>
+      <c r="F9" s="6"/>
+      <c r="G9" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H9" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>45</v>
+      </c>
+      <c r="B10" s="7">
+        <f>0.5711/0.777</f>
+        <v>0.73500643500643503</v>
+      </c>
+      <c r="C10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" t="s">
+        <v>21</v>
+      </c>
+      <c r="F10" s="6"/>
+      <c r="G10" t="s">
+        <v>20</v>
+      </c>
+      <c r="H10" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>170</v>
+      </c>
+      <c r="B11" s="4">
+        <f>2.1435</f>
+        <v>2.1435</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11" t="s">
+        <v>19</v>
+      </c>
+      <c r="E11" t="s">
+        <v>9</v>
+      </c>
+      <c r="G11" t="s">
+        <v>20</v>
+      </c>
+      <c r="H11" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>172</v>
+      </c>
+      <c r="B12" s="4">
+        <f>2.6847*3.6</f>
+        <v>9.6649200000000004</v>
+      </c>
+      <c r="C12" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12" t="s">
+        <v>4</v>
+      </c>
+      <c r="E12" t="s">
+        <v>23</v>
+      </c>
+      <c r="G12" t="s">
+        <v>20</v>
+      </c>
+      <c r="H12" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>53</v>
+      </c>
+      <c r="B13" s="4">
+        <f>0.00501</f>
+        <v>5.0099999999999997E-3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D13" t="s">
+        <v>42</v>
+      </c>
+      <c r="E13" t="s">
+        <v>24</v>
+      </c>
+      <c r="G13" t="s">
+        <v>20</v>
+      </c>
+      <c r="H13" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>53</v>
+      </c>
+      <c r="B14" s="4">
+        <v>0.30630000000000002</v>
+      </c>
+      <c r="C14" t="s">
+        <v>18</v>
+      </c>
+      <c r="D14" t="s">
+        <v>42</v>
+      </c>
+      <c r="E14" t="s">
+        <v>24</v>
+      </c>
+      <c r="G14" t="s">
+        <v>20</v>
+      </c>
+      <c r="H14" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>172</v>
+      </c>
+      <c r="B15" s="4">
+        <f>0.7493*3.6</f>
+        <v>2.6974800000000001</v>
+      </c>
+      <c r="C15" t="s">
+        <v>18</v>
+      </c>
+      <c r="D15" t="s">
+        <v>4</v>
+      </c>
+      <c r="E15" t="s">
+        <v>23</v>
+      </c>
+      <c r="G15" t="s">
+        <v>20</v>
+      </c>
+      <c r="H15" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A16" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="B16" s="11">
+        <f>0.047321*3.6</f>
+        <v>0.17035560000000002</v>
+      </c>
+      <c r="C16" t="s">
+        <v>18</v>
+      </c>
+      <c r="D16" t="s">
+        <v>19</v>
+      </c>
+      <c r="E16" t="s">
+        <v>23</v>
+      </c>
+      <c r="G16" t="s">
+        <v>20</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="B17" s="4">
+        <f>0.7508*3.6</f>
+        <v>2.7028799999999999</v>
+      </c>
+      <c r="C17" t="s">
+        <v>18</v>
+      </c>
+      <c r="D17" t="s">
+        <v>19</v>
+      </c>
+      <c r="E17" t="s">
+        <v>23</v>
+      </c>
+      <c r="G17" t="s">
+        <v>20</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>172</v>
+      </c>
+      <c r="B18" s="4">
+        <f>0.8098*3.6</f>
+        <v>2.9152800000000001</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18" t="s">
+        <v>4</v>
+      </c>
+      <c r="E18" t="s">
+        <v>23</v>
+      </c>
+      <c r="G18" t="s">
+        <v>20</v>
+      </c>
+      <c r="H18" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>29</v>
+      </c>
+      <c r="B19" s="4">
+        <v>0.35610000000000003</v>
+      </c>
+      <c r="C19" t="s">
+        <v>30</v>
+      </c>
+      <c r="E19" t="s">
+        <v>9</v>
+      </c>
+      <c r="F19" t="s">
+        <v>39</v>
+      </c>
+      <c r="G19" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20" s="13">
+        <f>0.8382/1000</f>
+        <v>8.3819999999999999E-4</v>
+      </c>
+      <c r="C20" t="s">
+        <v>30</v>
+      </c>
+      <c r="E20" t="s">
+        <v>21</v>
+      </c>
+      <c r="F20" t="s">
+        <v>39</v>
+      </c>
+      <c r="G20" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>36</v>
+      </c>
+      <c r="B21" s="4">
+        <v>3.9666000000000001</v>
+      </c>
+      <c r="C21" t="s">
+        <v>30</v>
+      </c>
+      <c r="E21" t="s">
+        <v>9</v>
+      </c>
+      <c r="F21" t="s">
+        <v>39</v>
+      </c>
+      <c r="G21" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>174</v>
+      </c>
+      <c r="B22" s="4">
+        <v>0.19411999999999999</v>
+      </c>
+      <c r="C22" t="s">
+        <v>30</v>
+      </c>
+      <c r="E22" t="s">
+        <v>9</v>
+      </c>
+      <c r="F22" t="s">
+        <v>39</v>
+      </c>
+      <c r="G22" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>38</v>
+      </c>
+      <c r="B23" s="11">
+        <f>1.3003/1000</f>
+        <v>1.3003000000000001E-3</v>
+      </c>
+      <c r="C23" t="s">
+        <v>30</v>
+      </c>
+      <c r="E23" t="s">
+        <v>21</v>
+      </c>
+      <c r="F23" t="s">
+        <v>40</v>
+      </c>
+      <c r="G23" t="s">
+        <v>31</v>
+      </c>
+      <c r="H23" s="12"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>175</v>
+      </c>
+      <c r="B24" s="4">
+        <v>1.4939E-3</v>
+      </c>
+      <c r="C24" t="s">
+        <v>30</v>
+      </c>
+      <c r="E24" t="s">
+        <v>9</v>
+      </c>
+      <c r="F24" t="s">
+        <v>39</v>
+      </c>
+      <c r="G24" t="s">
+        <v>31</v>
+      </c>
+      <c r="H24" s="12"/>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>98</v>
+      </c>
+      <c r="B25" s="13">
+        <f>0.0000058317+0.000023251</f>
+        <v>2.9082700000000002E-5</v>
+      </c>
+      <c r="C25" t="s">
+        <v>30</v>
+      </c>
+      <c r="E25" t="s">
+        <v>9</v>
+      </c>
+      <c r="F25" t="s">
+        <v>39</v>
+      </c>
+      <c r="G25" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>34</v>
+      </c>
+      <c r="B26" s="13">
+        <f>0.000000089737+0.0000047831</f>
+        <v>4.8728369999999997E-6</v>
+      </c>
+      <c r="C26" t="s">
+        <v>30</v>
+      </c>
+      <c r="E26" t="s">
+        <v>9</v>
+      </c>
+      <c r="F26" t="s">
+        <v>39</v>
+      </c>
+      <c r="G26" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>29</v>
+      </c>
+      <c r="B27" s="13">
+        <f>0.00082927+0.00042085</f>
+        <v>1.25012E-3</v>
+      </c>
+      <c r="C27" t="s">
+        <v>30</v>
+      </c>
+      <c r="E27" t="s">
+        <v>9</v>
+      </c>
+      <c r="F27" t="s">
+        <v>39</v>
+      </c>
+      <c r="G27" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="B28" s="13">
+        <f>(0.0000000026445+0.0000000000012752)/1000</f>
+        <v>2.6457752000000001E-12</v>
+      </c>
+      <c r="C28" t="s">
+        <v>30</v>
+      </c>
+      <c r="E28" t="s">
+        <v>21</v>
+      </c>
+      <c r="F28" t="s">
+        <v>39</v>
+      </c>
+      <c r="G28" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>36</v>
+      </c>
+      <c r="B29" s="13">
+        <f>0.0000017712+0.000015159</f>
+        <v>1.6930199999999999E-5</v>
+      </c>
+      <c r="C29" t="s">
+        <v>30</v>
+      </c>
+      <c r="E29" t="s">
+        <v>9</v>
+      </c>
+      <c r="F29" t="s">
+        <v>39</v>
+      </c>
+      <c r="G29" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>175</v>
+      </c>
+      <c r="B30" s="13">
+        <v>1.0015E-5</v>
+      </c>
+      <c r="C30" t="s">
+        <v>30</v>
+      </c>
+      <c r="E30" t="s">
+        <v>9</v>
+      </c>
+      <c r="F30" t="s">
+        <v>40</v>
+      </c>
+      <c r="G30" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>38</v>
+      </c>
+      <c r="B31" s="11">
+        <f>0.2644/1000</f>
+        <v>2.6440000000000003E-4</v>
+      </c>
+      <c r="C31" t="s">
+        <v>30</v>
+      </c>
+      <c r="E31" t="s">
+        <v>21</v>
+      </c>
+      <c r="F31" t="s">
+        <v>40</v>
+      </c>
+      <c r="G31" t="s">
+        <v>31</v>
+      </c>
+      <c r="H31" s="12"/>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>36</v>
+      </c>
+      <c r="B32" s="13">
+        <f>8.4573E-17</f>
+        <v>8.4573000000000001E-17</v>
+      </c>
+      <c r="C32" t="s">
+        <v>30</v>
+      </c>
+      <c r="E32" t="s">
+        <v>9</v>
+      </c>
+      <c r="F32" t="s">
+        <v>40</v>
+      </c>
+      <c r="G32" t="s">
+        <v>31</v>
+      </c>
+      <c r="H32" s="12"/>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" s="2"/>
+      <c r="B33" s="2"/>
+      <c r="C33" s="3"/>
+      <c r="D33" s="2"/>
+      <c r="E33" s="2"/>
+      <c r="F33" s="2"/>
+      <c r="G33" s="2"/>
+      <c r="H33" s="2"/>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="C34" s="6"/>
+      <c r="D34" s="6"/>
+      <c r="E34" s="6"/>
+      <c r="F34" s="6"/>
+      <c r="G34" s="6"/>
+      <c r="H34" s="6"/>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="B35" t="s">
+        <v>177</v>
+      </c>
+      <c r="C35" s="6"/>
+      <c r="D35" s="6"/>
+      <c r="E35" s="6"/>
+      <c r="F35" s="6"/>
+      <c r="G35" s="6"/>
+      <c r="H35" s="6"/>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A36" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B36" t="s">
+        <v>4</v>
+      </c>
+      <c r="C36" s="6"/>
+      <c r="D36" s="6"/>
+      <c r="E36" s="6"/>
+      <c r="F36" s="6"/>
+      <c r="G36" s="6"/>
+      <c r="H36" s="6"/>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A37" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B37" s="6">
+        <v>1</v>
+      </c>
+      <c r="C37" s="6"/>
+      <c r="D37" s="6"/>
+      <c r="E37" s="6"/>
+      <c r="F37" s="6"/>
+      <c r="G37" s="6"/>
+      <c r="H37" s="6"/>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A38" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B38" t="s">
+        <v>169</v>
+      </c>
+      <c r="C38" s="6"/>
+      <c r="D38" s="6"/>
+      <c r="E38" s="6"/>
+      <c r="F38" s="6"/>
+      <c r="G38" s="6"/>
+      <c r="H38" s="6"/>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A39" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B39" t="s">
+        <v>9</v>
+      </c>
+      <c r="C39" s="6"/>
+      <c r="D39" s="6"/>
+      <c r="E39" s="6"/>
+      <c r="F39" s="6"/>
+      <c r="G39" s="6"/>
+      <c r="H39" s="6"/>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A40" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B40" s="6"/>
+      <c r="C40" s="6"/>
+      <c r="D40" s="6"/>
+      <c r="E40" s="6"/>
+      <c r="F40" s="6"/>
+      <c r="G40" s="6"/>
+      <c r="H40" s="6"/>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A41" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D41" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E41" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F41" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="G41" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H41" s="6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>176</v>
+      </c>
+      <c r="B42" s="7">
+        <v>1</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D42" t="s">
+        <v>4</v>
+      </c>
+      <c r="E42" t="s">
+        <v>9</v>
+      </c>
+      <c r="F42" s="6"/>
+      <c r="G42" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H42" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>45</v>
+      </c>
+      <c r="B43" s="7">
+        <f>0.5711/0.777</f>
+        <v>0.73500643500643503</v>
+      </c>
+      <c r="C43" t="s">
+        <v>18</v>
+      </c>
+      <c r="D43" t="s">
+        <v>19</v>
+      </c>
+      <c r="E43" t="s">
+        <v>21</v>
+      </c>
+      <c r="F43" s="6"/>
+      <c r="G43" t="s">
+        <v>20</v>
+      </c>
+      <c r="H43" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>170</v>
+      </c>
+      <c r="B44" s="4">
+        <f>2.1435</f>
+        <v>2.1435</v>
+      </c>
+      <c r="C44" t="s">
+        <v>18</v>
+      </c>
+      <c r="D44" t="s">
+        <v>19</v>
+      </c>
+      <c r="E44" t="s">
+        <v>9</v>
+      </c>
+      <c r="G44" t="s">
+        <v>20</v>
+      </c>
+      <c r="H44" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>172</v>
+      </c>
+      <c r="B45" s="4">
+        <f>2.6847*3.6</f>
+        <v>9.6649200000000004</v>
+      </c>
+      <c r="C45" t="s">
+        <v>18</v>
+      </c>
+      <c r="D45" t="s">
+        <v>4</v>
+      </c>
+      <c r="E45" t="s">
+        <v>23</v>
+      </c>
+      <c r="G45" t="s">
+        <v>20</v>
+      </c>
+      <c r="H45" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>53</v>
+      </c>
+      <c r="B46" s="4">
+        <f>0.00501</f>
+        <v>5.0099999999999997E-3</v>
+      </c>
+      <c r="C46" t="s">
+        <v>18</v>
+      </c>
+      <c r="D46" t="s">
+        <v>42</v>
+      </c>
+      <c r="E46" t="s">
+        <v>24</v>
+      </c>
+      <c r="G46" t="s">
+        <v>20</v>
+      </c>
+      <c r="H46" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>53</v>
+      </c>
+      <c r="B47" s="4">
+        <v>0.30630000000000002</v>
+      </c>
+      <c r="C47" t="s">
+        <v>18</v>
+      </c>
+      <c r="D47" t="s">
+        <v>42</v>
+      </c>
+      <c r="E47" t="s">
+        <v>24</v>
+      </c>
+      <c r="G47" t="s">
+        <v>20</v>
+      </c>
+      <c r="H47" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>172</v>
+      </c>
+      <c r="B48" s="4">
+        <f>0.7493*3.6</f>
+        <v>2.6974800000000001</v>
+      </c>
+      <c r="C48" t="s">
+        <v>18</v>
+      </c>
+      <c r="D48" t="s">
+        <v>4</v>
+      </c>
+      <c r="E48" t="s">
+        <v>23</v>
+      </c>
+      <c r="G48" t="s">
+        <v>20</v>
+      </c>
+      <c r="H48" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A49" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="B49" s="11">
+        <f>0.047321*3.6</f>
+        <v>0.17035560000000002</v>
+      </c>
+      <c r="C49" t="s">
+        <v>18</v>
+      </c>
+      <c r="D49" t="s">
+        <v>4</v>
+      </c>
+      <c r="E49" t="s">
+        <v>23</v>
+      </c>
+      <c r="G49" t="s">
+        <v>20</v>
+      </c>
+      <c r="H49" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A50" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="B50" s="4">
+        <f>0.7508*3.6</f>
+        <v>2.7028799999999999</v>
+      </c>
+      <c r="C50" t="s">
+        <v>18</v>
+      </c>
+      <c r="D50" t="s">
+        <v>4</v>
+      </c>
+      <c r="E50" t="s">
+        <v>23</v>
+      </c>
+      <c r="G50" t="s">
+        <v>20</v>
+      </c>
+      <c r="H50" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>172</v>
+      </c>
+      <c r="B51" s="4">
+        <f>0.8098*3.6</f>
+        <v>2.9152800000000001</v>
+      </c>
+      <c r="C51" t="s">
+        <v>18</v>
+      </c>
+      <c r="D51" t="s">
+        <v>4</v>
+      </c>
+      <c r="E51" t="s">
+        <v>23</v>
+      </c>
+      <c r="G51" t="s">
+        <v>20</v>
+      </c>
+      <c r="H51" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>29</v>
+      </c>
+      <c r="B52" s="4">
+        <v>0.35610000000000003</v>
+      </c>
+      <c r="C52" t="s">
+        <v>30</v>
+      </c>
+      <c r="E52" t="s">
+        <v>9</v>
+      </c>
+      <c r="F52" t="s">
+        <v>39</v>
+      </c>
+      <c r="G52" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A53" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="B53" s="13">
+        <f>0.8382/1000</f>
+        <v>8.3819999999999999E-4</v>
+      </c>
+      <c r="C53" t="s">
+        <v>30</v>
+      </c>
+      <c r="E53" t="s">
+        <v>21</v>
+      </c>
+      <c r="F53" t="s">
+        <v>39</v>
+      </c>
+      <c r="G53" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>36</v>
+      </c>
+      <c r="B54" s="4">
+        <v>3.9666000000000001</v>
+      </c>
+      <c r="C54" t="s">
+        <v>30</v>
+      </c>
+      <c r="E54" t="s">
+        <v>9</v>
+      </c>
+      <c r="F54" t="s">
+        <v>39</v>
+      </c>
+      <c r="G54" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>174</v>
+      </c>
+      <c r="B55" s="4">
+        <v>0.19411999999999999</v>
+      </c>
+      <c r="C55" t="s">
+        <v>30</v>
+      </c>
+      <c r="E55" t="s">
+        <v>9</v>
+      </c>
+      <c r="F55" t="s">
+        <v>39</v>
+      </c>
+      <c r="G55" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>38</v>
+      </c>
+      <c r="B56" s="11">
+        <f>1.3003/1000</f>
+        <v>1.3003000000000001E-3</v>
+      </c>
+      <c r="C56" t="s">
+        <v>30</v>
+      </c>
+      <c r="E56" t="s">
+        <v>21</v>
+      </c>
+      <c r="F56" t="s">
+        <v>40</v>
+      </c>
+      <c r="G56" t="s">
+        <v>31</v>
+      </c>
+      <c r="H56" s="12"/>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>175</v>
+      </c>
+      <c r="B57" s="4">
+        <v>1.4939E-3</v>
+      </c>
+      <c r="C57" t="s">
+        <v>30</v>
+      </c>
+      <c r="E57" t="s">
+        <v>9</v>
+      </c>
+      <c r="F57" t="s">
+        <v>39</v>
+      </c>
+      <c r="G57" t="s">
+        <v>31</v>
+      </c>
+      <c r="H57" s="12"/>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>98</v>
+      </c>
+      <c r="B58" s="13">
+        <f>0.0000058317+0.000023251</f>
+        <v>2.9082700000000002E-5</v>
+      </c>
+      <c r="C58" t="s">
+        <v>30</v>
+      </c>
+      <c r="E58" t="s">
+        <v>9</v>
+      </c>
+      <c r="F58" t="s">
+        <v>39</v>
+      </c>
+      <c r="G58" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>34</v>
+      </c>
+      <c r="B59" s="13">
+        <f>0.000000089737+0.0000047831</f>
+        <v>4.8728369999999997E-6</v>
+      </c>
+      <c r="C59" t="s">
+        <v>30</v>
+      </c>
+      <c r="E59" t="s">
+        <v>9</v>
+      </c>
+      <c r="F59" t="s">
+        <v>39</v>
+      </c>
+      <c r="G59" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>29</v>
+      </c>
+      <c r="B60" s="13">
+        <f>0.00082927+0.00042085</f>
+        <v>1.25012E-3</v>
+      </c>
+      <c r="C60" t="s">
+        <v>30</v>
+      </c>
+      <c r="E60" t="s">
+        <v>9</v>
+      </c>
+      <c r="F60" t="s">
+        <v>39</v>
+      </c>
+      <c r="G60" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A61" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="B61" s="13">
+        <f>(0.0000000026445+0.0000000000012752)/1000</f>
+        <v>2.6457752000000001E-12</v>
+      </c>
+      <c r="C61" t="s">
+        <v>30</v>
+      </c>
+      <c r="E61" t="s">
+        <v>21</v>
+      </c>
+      <c r="F61" t="s">
+        <v>39</v>
+      </c>
+      <c r="G61" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>36</v>
+      </c>
+      <c r="B62" s="13">
+        <f>0.0000017712+0.000015159</f>
+        <v>1.6930199999999999E-5</v>
+      </c>
+      <c r="C62" t="s">
+        <v>30</v>
+      </c>
+      <c r="E62" t="s">
+        <v>9</v>
+      </c>
+      <c r="F62" t="s">
+        <v>39</v>
+      </c>
+      <c r="G62" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>175</v>
+      </c>
+      <c r="B63" s="13">
+        <v>1.0015E-5</v>
+      </c>
+      <c r="C63" t="s">
+        <v>30</v>
+      </c>
+      <c r="E63" t="s">
+        <v>9</v>
+      </c>
+      <c r="F63" t="s">
+        <v>40</v>
+      </c>
+      <c r="G63" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>38</v>
+      </c>
+      <c r="B64" s="11">
+        <f>0.2644/1000</f>
+        <v>2.6440000000000003E-4</v>
+      </c>
+      <c r="C64" t="s">
+        <v>30</v>
+      </c>
+      <c r="E64" t="s">
+        <v>21</v>
+      </c>
+      <c r="F64" t="s">
+        <v>40</v>
+      </c>
+      <c r="G64" t="s">
+        <v>31</v>
+      </c>
+      <c r="H64" s="12"/>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>36</v>
+      </c>
+      <c r="B65" s="13">
+        <f>8.4573E-17</f>
+        <v>8.4573000000000001E-17</v>
+      </c>
+      <c r="C65" t="s">
+        <v>30</v>
+      </c>
+      <c r="E65" t="s">
+        <v>9</v>
+      </c>
+      <c r="F65" t="s">
+        <v>40</v>
+      </c>
+      <c r="G65" t="s">
+        <v>31</v>
+      </c>
+      <c r="H65" s="12"/>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A66" s="6"/>
+      <c r="B66" s="11"/>
+      <c r="C66" s="6"/>
+      <c r="D66" s="6"/>
+      <c r="E66" s="6"/>
+      <c r="F66" s="6"/>
+      <c r="H66" s="6"/>
+    </row>
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A77" s="6"/>
+      <c r="B77" s="4"/>
+      <c r="C77" s="6"/>
+      <c r="F77" s="6"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>